<commit_message>
Fis bug with receive rreg packet
</commit_message>
<xml_diff>
--- a/debug.xlsx
+++ b/debug.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="State" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -709,11 +709,11 @@
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 32];
-rreg: trgt-23:[31, 34];
-rreg: trgt-23:[31, 37];
-rreg: trgt-23:[31, 46];
-rreg: trgt-23:[31, 44];
+          <t xml:space="preserve">rreg:[31, 32];
+rreg:[31, 34];
+rreg:[31, 37];
+rreg:[31, 46];
+rreg:[31, 44];
 </t>
         </is>
       </c>
@@ -840,17 +840,17 @@
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 32, 34];
+          <t xml:space="preserve">rreg:[31, 32, 34];
 </t>
         </is>
       </c>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 34, 32];
-rreg: trgt-23:[31, 34, 46];
-rreg: trgt-23:[31, 34, 35];
-rreg: trgt-23:[31, 34, 44];
+          <t xml:space="preserve">rreg:[31, 34, 32];
+rreg:[31, 34, 46];
+rreg:[31, 34, 35];
+rreg:[31, 34, 44];
 </t>
         </is>
       </c>
@@ -858,8 +858,8 @@
       <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 44];
-rreg: trgt-23:[31, 37, 40];
+          <t xml:space="preserve">rreg:[31, 37, 44];
+rreg:[31, 37, 40];
 </t>
         </is>
       </c>
@@ -871,19 +871,19 @@
       <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 44, 34];
-rreg: trgt-23:[31, 44, 36];
-rreg: trgt-23:[31, 44, 37];
+          <t xml:space="preserve">rreg:[31, 44, 34];
+rreg:[31, 44, 36];
+rreg:[31, 44, 37];
 </t>
         </is>
       </c>
       <c r="AU6" t="inlineStr"/>
       <c r="AV6" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 3];
-rreg: trgt-23:[31, 46, 7];
-rreg: trgt-23:[31, 46, 11];
-rreg: trgt-23:[31, 46, 34];
+          <t xml:space="preserve">rreg:[31, 46, 3];
+rreg:[31, 46, 7];
+rreg:[31, 46, 11];
+rreg:[31, 46, 34];
 </t>
         </is>
       </c>
@@ -966,10 +966,10 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 3, 41];
-rreg: trgt-23:[31, 46, 3, 17];
-rreg: trgt-23:[31, 46, 3, 19];
-rreg: trgt-23:[31, 46, 3, 28];
+          <t xml:space="preserve">rreg:[31, 46, 3, 41];
+rreg:[31, 46, 3, 17];
+rreg:[31, 46, 3, 19];
+rreg:[31, 46, 3, 28];
 </t>
         </is>
       </c>
@@ -978,7 +978,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 7, 28];
+          <t xml:space="preserve">rreg:[31, 46, 7, 28];
 </t>
         </is>
       </c>
@@ -987,10 +987,10 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 11, 28];
-rreg: trgt-23:[31, 46, 11, 41];
-rreg: trgt-23:[31, 46, 11, 30];
-rreg: trgt-23:[31, 46, 11, 29];
+          <t xml:space="preserve">rreg:[31, 46, 11, 28];
+rreg:[31, 46, 11, 41];
+rreg:[31, 46, 11, 30];
+rreg:[31, 46, 11, 29];
 </t>
         </is>
       </c>
@@ -1019,13 +1019,13 @@
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 34, 35, 0];
+          <t xml:space="preserve">rreg:[31, 34, 35, 0];
 </t>
         </is>
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 44, 36, 0];
+          <t xml:space="preserve">rreg:[31, 44, 36, 0];
 </t>
         </is>
       </c>
@@ -1034,7 +1034,7 @@
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22];
 </t>
         </is>
       </c>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 44, 36, 0, 35];
+          <t xml:space="preserve">rreg:[31, 44, 36, 0, 35];
 </t>
         </is>
       </c>
@@ -1142,14 +1142,14 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 3, 17, 19];
+          <t xml:space="preserve">rreg:[31, 46, 3, 17, 19];
 </t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 3, 19, 17];
+          <t xml:space="preserve">rreg:[31, 46, 3, 19, 17];
 </t>
         </is>
       </c>
@@ -1157,10 +1157,10 @@
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5];
-rreg: trgt-23:[31, 37, 40, 22, 8];
-rreg: trgt-23:[31, 37, 40, 22, 18];
-rreg: trgt-23:[31, 37, 40, 22, 21];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+rreg:[31, 37, 40, 22, 18];
+rreg:[31, 37, 40, 22, 21];
 </t>
         </is>
       </c>
@@ -1171,23 +1171,23 @@
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 3, 28, 7];
-rreg: trgt-23:[31, 46, 3, 28, 11];
-rreg: trgt-23:[31, 46, 3, 28, 41];
-rreg: trgt-23:[31, 46, 3, 28, 30];
+          <t xml:space="preserve">rreg:[31, 46, 3, 28, 7];
+rreg:[31, 46, 3, 28, 11];
+rreg:[31, 46, 3, 28, 41];
+rreg:[31, 46, 3, 28, 30];
 </t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 11, 29, 18];
+          <t xml:space="preserve">rreg:[31, 46, 11, 29, 18];
 </t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 11, 30, 28];
-rreg: trgt-23:[31, 46, 11, 30, 41];
+          <t xml:space="preserve">rreg:[31, 46, 11, 30, 28];
+rreg:[31, 46, 11, 30, 41];
 </t>
         </is>
       </c>
@@ -1203,9 +1203,9 @@
       <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 46, 3, 41, 11];
-rreg: trgt-23:[31, 46, 3, 41, 28];
-rreg: trgt-23:[31, 46, 3, 41, 30];
+          <t xml:space="preserve">rreg:[31, 46, 3, 41, 11];
+rreg:[31, 46, 3, 41, 28];
+rreg:[31, 46, 3, 41, 30];
 </t>
         </is>
       </c>
@@ -1295,10 +1295,10 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 18];
-rreg: trgt-23:[31, 37, 40, 22, 5, 24];
-rreg: trgt-23:[31, 37, 40, 22, 5, 39];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 18];
+rreg:[31, 37, 40, 22, 5, 24];
+rreg:[31, 37, 40, 22, 5, 39];
+rreg:[31, 37, 40, 22, 5, 45];
 </t>
         </is>
       </c>
@@ -1306,10 +1306,10 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 8, 24];
-rreg: trgt-23:[31, 37, 40, 22, 8, 47];
-rreg: trgt-23:[31, 37, 40, 22, 8, 39];
-rreg: trgt-23:[31, 37, 40, 22, 8, 21];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 8, 24];
+rreg:[31, 37, 40, 22, 8, 47];
+rreg:[31, 37, 40, 22, 8, 39];
+rreg:[31, 37, 40, 22, 8, 21];
 </t>
         </is>
       </c>
@@ -1324,10 +1324,10 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 18, 5];
-rreg: trgt-23:[31, 37, 40, 22, 18, 45];
-rreg: trgt-23:[31, 37, 40, 22, 18, 29];
-rreg: trgt-23:[31, 37, 40, 22, 18, 21];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+rreg:[31, 37, 40, 22, 18, 45];
+rreg:[31, 37, 40, 22, 18, 29];
+rreg:[31, 37, 40, 22, 18, 21];
 </t>
         </is>
       </c>
@@ -1335,8 +1335,8 @@
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 21, 8];
-rreg: trgt-23:[31, 37, 40, 22, 21, 18];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8];
+rreg:[31, 37, 40, 22, 21, 18];
 </t>
         </is>
       </c>
@@ -1465,7 +1465,7 @@
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 24, 8];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 24, 8];
 </t>
         </is>
       </c>
@@ -1485,9 +1485,9 @@
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 39, 8];
-rreg: trgt-23:[31, 37, 40, 22, 5, 39, 20];
-rreg: trgt-23:[31, 37, 40, 22, 5, 39, 42];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 39, 8];
+rreg:[31, 37, 40, 22, 5, 39, 20];
+rreg:[31, 37, 40, 22, 5, 39, 42];
 </t>
         </is>
       </c>
@@ -1498,17 +1498,17 @@
       <c r="AT18" t="inlineStr"/>
       <c r="AU18" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 2];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 9];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 18];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 2];
+rreg:[31, 37, 40, 22, 5, 45, 9];
+rreg:[31, 37, 40, 22, 5, 45, 18];
+rreg:[31, 37, 40, 22, 5, 45, 20];
 </t>
         </is>
       </c>
       <c r="AV18" t="inlineStr"/>
       <c r="AW18" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 8, 47, 4];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 8, 47, 4];
 </t>
         </is>
       </c>
@@ -1589,16 +1589,16 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 2, 9];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 2, 20];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 2, 9];
+rreg:[31, 37, 40, 22, 5, 45, 2, 20];
 </t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 8, 47, 4, 9];
-rreg: trgt-23:[31, 37, 40, 22, 8, 47, 4, 10];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 8, 47, 4, 9];
+rreg:[31, 37, 40, 22, 8, 47, 4, 10];
 </t>
         </is>
       </c>
@@ -1608,9 +1608,9 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 9, 2];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 9, 4];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 9, 27];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 9, 2];
+rreg:[31, 37, 40, 22, 5, 45, 9, 4];
+rreg:[31, 37, 40, 22, 5, 45, 9, 27];
 </t>
         </is>
       </c>
@@ -1626,10 +1626,10 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 2];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 27];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 39];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 2];
+rreg:[31, 37, 40, 22, 5, 45, 20, 27];
+rreg:[31, 37, 40, 22, 5, 45, 20, 38];
+rreg:[31, 37, 40, 22, 5, 45, 20, 39];
 </t>
         </is>
       </c>
@@ -1656,9 +1656,9 @@
       <c r="AQ21" t="inlineStr"/>
       <c r="AR21" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33];
-rreg: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43];
-rreg: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 39, 42, 33];
+rreg:[31, 37, 40, 22, 5, 39, 42, 43];
+rreg:[31, 37, 40, 22, 5, 39, 42, 43];
 </t>
         </is>
       </c>
@@ -1752,7 +1752,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 8, 47, 4, 10, 1];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 8, 47, 4, 10, 1];
 </t>
         </is>
       </c>
@@ -1774,8 +1774,8 @@
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 9, 27, 1];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 9, 27, 20];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 9, 27, 1];
+rreg:[31, 37, 40, 22, 5, 45, 9, 27, 20];
 </t>
         </is>
       </c>
@@ -1786,7 +1786,7 @@
       <c r="AH24" t="inlineStr"/>
       <c r="AI24" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -1796,8 +1796,8 @@
       <c r="AM24" t="inlineStr"/>
       <c r="AN24" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 12];
+rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15];
 </t>
         </is>
       </c>
@@ -1807,8 +1807,8 @@
       <c r="AR24" t="inlineStr"/>
       <c r="AS24" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43, 13];
-rreg: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43, 33];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 39, 42, 43, 13];
+rreg:[31, 37, 40, 22, 5, 39, 42, 43, 33];
 </t>
         </is>
       </c>
@@ -1892,7 +1892,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 9, 27, 1, 10];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 9, 27, 1, 10];
 </t>
         </is>
       </c>
@@ -1908,22 +1908,22 @@
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6];
+rreg:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26];
 </t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33];
 </t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 26];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15, 26];
+rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25];
 </t>
         </is>
       </c>
@@ -1946,7 +1946,7 @@
       <c r="AH27" t="inlineStr"/>
       <c r="AI27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
 </t>
         </is>
       </c>
@@ -1960,7 +1960,7 @@
       <c r="AQ27" t="inlineStr"/>
       <c r="AR27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2050,7 +2050,7 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
 </t>
         </is>
       </c>
@@ -2074,14 +2074,14 @@
       <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6];
-rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 16];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6];
+rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 16];
 </t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15];
 </t>
         </is>
       </c>
@@ -2093,7 +2093,7 @@
       <c r="AH30" t="inlineStr"/>
       <c r="AI30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33, 23];
 </t>
         </is>
       </c>
@@ -2104,9 +2104,9 @@
       <c r="AN30" t="inlineStr"/>
       <c r="AO30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 8, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2115,8 +2115,8 @@
       <c r="AR30" t="inlineStr"/>
       <c r="AS30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
+rrep:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
 </t>
         </is>
       </c>
@@ -2204,24 +2204,24 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
 </t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 8, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 24, 8, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 39, 8, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 24, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 39, 8, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2230,13 +2230,13 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
 </t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33, 23];
 </t>
         </is>
       </c>
@@ -2244,7 +2244,7 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 16, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 16, 23];
 </t>
         </is>
       </c>
@@ -2253,10 +2253,10 @@
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 39, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 2, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 9, 27, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 39, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 2, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 9, 27, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2364,9 +2364,9 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 2, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 9, 2, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 2, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 2, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 9, 2, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 20, 2, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2387,11 +2387,11 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 21, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 18, 5, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 18, 5, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2399,37 +2399,37 @@
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 8, 21, 8, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 18, 21, 8, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 21, 8, 39, 42, 33, 23];
 </t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
       <c r="Y36" t="inlineStr"/>
       <c r="Z36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 24, 8, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 8, 24, 8, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 24, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 24, 8, 39, 42, 33, 23];
 </t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
 </t>
         </is>
       </c>
       <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 9, 27, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 27, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 9, 27, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 20, 27, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2445,7 +2445,7 @@
       <c r="AM36" t="inlineStr"/>
       <c r="AN36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
 </t>
         </is>
       </c>
@@ -2457,8 +2457,8 @@
       <c r="AT36" t="inlineStr"/>
       <c r="AU36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 18, 45, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2548,9 +2548,9 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 9, 2, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 2, 9, 2, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 9, 2, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 2, 9, 2, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2561,8 +2561,8 @@
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15, 25, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
+rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15, 25, 6, 23];
 </t>
         </is>
       </c>
@@ -2581,8 +2581,8 @@
       <c r="AD39" t="inlineStr"/>
       <c r="AE39" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 18, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2598,7 +2598,7 @@
       <c r="AO39" t="inlineStr"/>
       <c r="AP39" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2688,8 +2688,8 @@
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 9, 4, 9, 2, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 5, 45, 9, 4, 9, 2, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2701,9 +2701,9 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 3, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 3, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2723,8 +2723,8 @@
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15, 25, 6, 23];
-rrep: trgt-23:[31, 37, 40, 22, 5, 45, 20, 38, 15, 26, 15, 25, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15, 25, 6, 23];
+rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 26, 15, 25, 6, 23];
 </t>
         </is>
       </c>
@@ -2740,8 +2740,8 @@
       <c r="AL42" t="inlineStr"/>
       <c r="AM42" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 44, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+rrep:[31, 44, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2858,11 +2858,11 @@
       <c r="AC45" t="inlineStr"/>
       <c r="AD45" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 46, 3, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 11, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 3, 41, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 11, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 46, 3, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 11, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 3, 41, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 11, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2870,7 +2870,7 @@
       <c r="AF45" t="inlineStr"/>
       <c r="AG45" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2885,10 +2885,10 @@
       <c r="AP45" t="inlineStr"/>
       <c r="AQ45" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 11, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 3, 28, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 11, 30, 41, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 11, 41, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 3, 28, 41, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 11, 30, 41, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2896,23 +2896,23 @@
       <c r="AS45" t="inlineStr"/>
       <c r="AT45" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 44, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 34, 44, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 37, 44, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 44, 37, 40, 22, 5, 39, 42, 33, 23];
+rrep:[31, 34, 44, 37, 40, 22, 5, 39, 42, 33, 23];
+rrep:[31, 37, 44, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
       <c r="AU45" t="inlineStr"/>
       <c r="AV45" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
       <c r="AW45" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2990,7 +2990,7 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2999,8 +2999,8 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 46, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 3, 28, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 46, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 3, 28, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3028,9 +3028,9 @@
       <c r="AE48" t="inlineStr"/>
       <c r="AF48" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 46, 11, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 3, 28, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 3, 41, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 46, 11, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 3, 28, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 3, 41, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3039,10 +3039,10 @@
       <c r="AI48" t="inlineStr"/>
       <c r="AJ48" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 46, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 44, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 46, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 44, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3050,7 +3050,7 @@
       <c r="AL48" t="inlineStr"/>
       <c r="AM48" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3167,8 +3167,8 @@
       <c r="AG51" t="inlineStr"/>
       <c r="AH51" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep: trgt-23:[31, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep: trgt-23:[31, 34, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
+rrep:[31, 34, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3178,7 +3178,7 @@
       <c r="AL51" t="inlineStr"/>
       <c r="AM51" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3300,7 +3300,7 @@
       <c r="AL54" t="inlineStr"/>
       <c r="AM54" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3422,7 +3422,7 @@
       <c r="AL57" t="inlineStr"/>
       <c r="AM57" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3544,7 +3544,7 @@
       <c r="AL60" t="inlineStr"/>
       <c r="AM60" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3666,7 +3666,7 @@
       <c r="AL63" t="inlineStr"/>
       <c r="AM63" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3788,7 +3788,7 @@
       <c r="AL66" t="inlineStr"/>
       <c r="AM66" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -3910,7 +3910,7 @@
       <c r="AL69" t="inlineStr"/>
       <c r="AM69" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -4032,7 +4032,7 @@
       <c r="AL72" t="inlineStr"/>
       <c r="AM72" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -4154,7 +4154,7 @@
       <c r="AL75" t="inlineStr"/>
       <c r="AM75" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -4276,7 +4276,7 @@
       <c r="AL78" t="inlineStr"/>
       <c r="AM78" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -4398,7 +4398,7 @@
       <c r="AL81" t="inlineStr"/>
       <c r="AM81" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -4520,7 +4520,7 @@
       <c r="AL84" t="inlineStr"/>
       <c r="AM84" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -4642,7 +4642,7 @@
       <c r="AL87" t="inlineStr"/>
       <c r="AM87" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -4764,7 +4764,7 @@
       <c r="AL90" t="inlineStr"/>
       <c r="AM90" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -4886,7 +4886,7 @@
       <c r="AL93" t="inlineStr"/>
       <c r="AM93" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5008,7 +5008,7 @@
       <c r="AL96" t="inlineStr"/>
       <c r="AM96" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5130,7 +5130,7 @@
       <c r="AL99" t="inlineStr"/>
       <c r="AM99" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5252,7 +5252,7 @@
       <c r="AL102" t="inlineStr"/>
       <c r="AM102" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5374,7 +5374,7 @@
       <c r="AL105" t="inlineStr"/>
       <c r="AM105" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5496,7 +5496,7 @@
       <c r="AL108" t="inlineStr"/>
       <c r="AM108" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5618,7 +5618,7 @@
       <c r="AL111" t="inlineStr"/>
       <c r="AM111" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5740,7 +5740,7 @@
       <c r="AL114" t="inlineStr"/>
       <c r="AM114" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5862,7 +5862,7 @@
       <c r="AL117" t="inlineStr"/>
       <c r="AM117" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -5984,7 +5984,7 @@
       <c r="AL120" t="inlineStr"/>
       <c r="AM120" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -6106,7 +6106,7 @@
       <c r="AL123" t="inlineStr"/>
       <c r="AM123" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -6228,7 +6228,7 @@
       <c r="AL126" t="inlineStr"/>
       <c r="AM126" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -6350,7 +6350,7 @@
       <c r="AL129" t="inlineStr"/>
       <c r="AM129" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -6472,7 +6472,7 @@
       <c r="AL132" t="inlineStr"/>
       <c r="AM132" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -6594,7 +6594,7 @@
       <c r="AL135" t="inlineStr"/>
       <c r="AM135" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -6716,7 +6716,7 @@
       <c r="AL138" t="inlineStr"/>
       <c r="AM138" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -6838,7 +6838,7 @@
       <c r="AL141" t="inlineStr"/>
       <c r="AM141" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -6960,7 +6960,7 @@
       <c r="AL144" t="inlineStr"/>
       <c r="AM144" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -7082,7 +7082,7 @@
       <c r="AL147" t="inlineStr"/>
       <c r="AM147" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -7204,7 +7204,7 @@
       <c r="AL150" t="inlineStr"/>
       <c r="AM150" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -7326,7 +7326,7 @@
       <c r="AL153" t="inlineStr"/>
       <c r="AM153" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -7448,7 +7448,7 @@
       <c r="AL156" t="inlineStr"/>
       <c r="AM156" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -7570,7 +7570,7 @@
       <c r="AL159" t="inlineStr"/>
       <c r="AM159" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -7692,7 +7692,7 @@
       <c r="AL162" t="inlineStr"/>
       <c r="AM162" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -7814,7 +7814,7 @@
       <c r="AL165" t="inlineStr"/>
       <c r="AM165" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -7936,7 +7936,7 @@
       <c r="AL168" t="inlineStr"/>
       <c r="AM168" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -8058,7 +8058,7 @@
       <c r="AL171" t="inlineStr"/>
       <c r="AM171" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -8180,7 +8180,7 @@
       <c r="AL174" t="inlineStr"/>
       <c r="AM174" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -8302,7 +8302,7 @@
       <c r="AL177" t="inlineStr"/>
       <c r="AM177" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -8424,7 +8424,7 @@
       <c r="AL180" t="inlineStr"/>
       <c r="AM180" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -8546,7 +8546,7 @@
       <c r="AL183" t="inlineStr"/>
       <c r="AM183" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -8668,7 +8668,7 @@
       <c r="AL186" t="inlineStr"/>
       <c r="AM186" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -8790,7 +8790,7 @@
       <c r="AL189" t="inlineStr"/>
       <c r="AM189" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -8912,7 +8912,7 @@
       <c r="AL192" t="inlineStr"/>
       <c r="AM192" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -9034,7 +9034,7 @@
       <c r="AL195" t="inlineStr"/>
       <c r="AM195" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -9156,7 +9156,7 @@
       <c r="AL198" t="inlineStr"/>
       <c r="AM198" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -9278,7 +9278,7 @@
       <c r="AL201" t="inlineStr"/>
       <c r="AM201" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -9400,7 +9400,7 @@
       <c r="AL204" t="inlineStr"/>
       <c r="AM204" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -9522,7 +9522,7 @@
       <c r="AL207" t="inlineStr"/>
       <c r="AM207" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -9644,7 +9644,7 @@
       <c r="AL210" t="inlineStr"/>
       <c r="AM210" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -9766,7 +9766,7 @@
       <c r="AL213" t="inlineStr"/>
       <c r="AM213" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -9888,7 +9888,7 @@
       <c r="AL216" t="inlineStr"/>
       <c r="AM216" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10010,7 +10010,7 @@
       <c r="AL219" t="inlineStr"/>
       <c r="AM219" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10132,7 +10132,7 @@
       <c r="AL222" t="inlineStr"/>
       <c r="AM222" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10254,7 +10254,7 @@
       <c r="AL225" t="inlineStr"/>
       <c r="AM225" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10376,7 +10376,7 @@
       <c r="AL228" t="inlineStr"/>
       <c r="AM228" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10498,7 +10498,7 @@
       <c r="AL231" t="inlineStr"/>
       <c r="AM231" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10620,7 +10620,7 @@
       <c r="AL234" t="inlineStr"/>
       <c r="AM234" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10742,7 +10742,7 @@
       <c r="AL237" t="inlineStr"/>
       <c r="AM237" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10864,7 +10864,7 @@
       <c r="AL240" t="inlineStr"/>
       <c r="AM240" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -10986,7 +10986,7 @@
       <c r="AL243" t="inlineStr"/>
       <c r="AM243" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -11108,7 +11108,7 @@
       <c r="AL246" t="inlineStr"/>
       <c r="AM246" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -11230,7 +11230,7 @@
       <c r="AL249" t="inlineStr"/>
       <c r="AM249" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -11352,7 +11352,7 @@
       <c r="AL252" t="inlineStr"/>
       <c r="AM252" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -11474,7 +11474,7 @@
       <c r="AL255" t="inlineStr"/>
       <c r="AM255" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -11596,7 +11596,7 @@
       <c r="AL258" t="inlineStr"/>
       <c r="AM258" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -11718,7 +11718,7 @@
       <c r="AL261" t="inlineStr"/>
       <c r="AM261" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -11840,7 +11840,7 @@
       <c r="AL264" t="inlineStr"/>
       <c r="AM264" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -11962,7 +11962,7 @@
       <c r="AL267" t="inlineStr"/>
       <c r="AM267" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -12084,7 +12084,7 @@
       <c r="AL270" t="inlineStr"/>
       <c r="AM270" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -12206,7 +12206,7 @@
       <c r="AL273" t="inlineStr"/>
       <c r="AM273" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -12328,7 +12328,7 @@
       <c r="AL276" t="inlineStr"/>
       <c r="AM276" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -12450,7 +12450,7 @@
       <c r="AL279" t="inlineStr"/>
       <c r="AM279" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -12572,7 +12572,7 @@
       <c r="AL282" t="inlineStr"/>
       <c r="AM282" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -12694,7 +12694,7 @@
       <c r="AL285" t="inlineStr"/>
       <c r="AM285" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -12816,7 +12816,7 @@
       <c r="AL288" t="inlineStr"/>
       <c r="AM288" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -12938,7 +12938,7 @@
       <c r="AL291" t="inlineStr"/>
       <c r="AM291" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -13060,7 +13060,7 @@
       <c r="AL294" t="inlineStr"/>
       <c r="AM294" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -13182,7 +13182,7 @@
       <c r="AL297" t="inlineStr"/>
       <c r="AM297" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -13304,7 +13304,7 @@
       <c r="AL300" t="inlineStr"/>
       <c r="AM300" t="inlineStr">
         <is>
-          <t xml:space="preserve">data: trgt-23:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add packet type check
</commit_message>
<xml_diff>
--- a/debug.xlsx
+++ b/debug.xlsx
@@ -3048,12 +3048,7 @@
       </c>
       <c r="AK48" t="inlineStr"/>
       <c r="AL48" t="inlineStr"/>
-      <c r="AM48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM48" t="inlineStr"/>
       <c r="AN48" t="inlineStr"/>
       <c r="AO48" t="inlineStr"/>
       <c r="AP48" t="inlineStr"/>
@@ -3176,12 +3171,7 @@
       <c r="AJ51" t="inlineStr"/>
       <c r="AK51" t="inlineStr"/>
       <c r="AL51" t="inlineStr"/>
-      <c r="AM51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM51" t="inlineStr"/>
       <c r="AN51" t="inlineStr"/>
       <c r="AO51" t="inlineStr"/>
       <c r="AP51" t="inlineStr"/>
@@ -3298,12 +3288,7 @@
       <c r="AJ54" t="inlineStr"/>
       <c r="AK54" t="inlineStr"/>
       <c r="AL54" t="inlineStr"/>
-      <c r="AM54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM54" t="inlineStr"/>
       <c r="AN54" t="inlineStr"/>
       <c r="AO54" t="inlineStr"/>
       <c r="AP54" t="inlineStr"/>
@@ -3420,12 +3405,7 @@
       <c r="AJ57" t="inlineStr"/>
       <c r="AK57" t="inlineStr"/>
       <c r="AL57" t="inlineStr"/>
-      <c r="AM57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM57" t="inlineStr"/>
       <c r="AN57" t="inlineStr"/>
       <c r="AO57" t="inlineStr"/>
       <c r="AP57" t="inlineStr"/>
@@ -3542,12 +3522,7 @@
       <c r="AJ60" t="inlineStr"/>
       <c r="AK60" t="inlineStr"/>
       <c r="AL60" t="inlineStr"/>
-      <c r="AM60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM60" t="inlineStr"/>
       <c r="AN60" t="inlineStr"/>
       <c r="AO60" t="inlineStr"/>
       <c r="AP60" t="inlineStr"/>
@@ -3664,12 +3639,7 @@
       <c r="AJ63" t="inlineStr"/>
       <c r="AK63" t="inlineStr"/>
       <c r="AL63" t="inlineStr"/>
-      <c r="AM63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM63" t="inlineStr"/>
       <c r="AN63" t="inlineStr"/>
       <c r="AO63" t="inlineStr"/>
       <c r="AP63" t="inlineStr"/>
@@ -3786,12 +3756,7 @@
       <c r="AJ66" t="inlineStr"/>
       <c r="AK66" t="inlineStr"/>
       <c r="AL66" t="inlineStr"/>
-      <c r="AM66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM66" t="inlineStr"/>
       <c r="AN66" t="inlineStr"/>
       <c r="AO66" t="inlineStr"/>
       <c r="AP66" t="inlineStr"/>
@@ -3908,12 +3873,7 @@
       <c r="AJ69" t="inlineStr"/>
       <c r="AK69" t="inlineStr"/>
       <c r="AL69" t="inlineStr"/>
-      <c r="AM69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM69" t="inlineStr"/>
       <c r="AN69" t="inlineStr"/>
       <c r="AO69" t="inlineStr"/>
       <c r="AP69" t="inlineStr"/>
@@ -4030,12 +3990,7 @@
       <c r="AJ72" t="inlineStr"/>
       <c r="AK72" t="inlineStr"/>
       <c r="AL72" t="inlineStr"/>
-      <c r="AM72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM72" t="inlineStr"/>
       <c r="AN72" t="inlineStr"/>
       <c r="AO72" t="inlineStr"/>
       <c r="AP72" t="inlineStr"/>
@@ -4152,12 +4107,7 @@
       <c r="AJ75" t="inlineStr"/>
       <c r="AK75" t="inlineStr"/>
       <c r="AL75" t="inlineStr"/>
-      <c r="AM75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM75" t="inlineStr"/>
       <c r="AN75" t="inlineStr"/>
       <c r="AO75" t="inlineStr"/>
       <c r="AP75" t="inlineStr"/>
@@ -4274,12 +4224,7 @@
       <c r="AJ78" t="inlineStr"/>
       <c r="AK78" t="inlineStr"/>
       <c r="AL78" t="inlineStr"/>
-      <c r="AM78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM78" t="inlineStr"/>
       <c r="AN78" t="inlineStr"/>
       <c r="AO78" t="inlineStr"/>
       <c r="AP78" t="inlineStr"/>
@@ -4396,12 +4341,7 @@
       <c r="AJ81" t="inlineStr"/>
       <c r="AK81" t="inlineStr"/>
       <c r="AL81" t="inlineStr"/>
-      <c r="AM81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM81" t="inlineStr"/>
       <c r="AN81" t="inlineStr"/>
       <c r="AO81" t="inlineStr"/>
       <c r="AP81" t="inlineStr"/>
@@ -4518,12 +4458,7 @@
       <c r="AJ84" t="inlineStr"/>
       <c r="AK84" t="inlineStr"/>
       <c r="AL84" t="inlineStr"/>
-      <c r="AM84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM84" t="inlineStr"/>
       <c r="AN84" t="inlineStr"/>
       <c r="AO84" t="inlineStr"/>
       <c r="AP84" t="inlineStr"/>
@@ -4640,12 +4575,7 @@
       <c r="AJ87" t="inlineStr"/>
       <c r="AK87" t="inlineStr"/>
       <c r="AL87" t="inlineStr"/>
-      <c r="AM87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM87" t="inlineStr"/>
       <c r="AN87" t="inlineStr"/>
       <c r="AO87" t="inlineStr"/>
       <c r="AP87" t="inlineStr"/>
@@ -4762,12 +4692,7 @@
       <c r="AJ90" t="inlineStr"/>
       <c r="AK90" t="inlineStr"/>
       <c r="AL90" t="inlineStr"/>
-      <c r="AM90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM90" t="inlineStr"/>
       <c r="AN90" t="inlineStr"/>
       <c r="AO90" t="inlineStr"/>
       <c r="AP90" t="inlineStr"/>
@@ -4884,12 +4809,7 @@
       <c r="AJ93" t="inlineStr"/>
       <c r="AK93" t="inlineStr"/>
       <c r="AL93" t="inlineStr"/>
-      <c r="AM93" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM93" t="inlineStr"/>
       <c r="AN93" t="inlineStr"/>
       <c r="AO93" t="inlineStr"/>
       <c r="AP93" t="inlineStr"/>
@@ -5006,12 +4926,7 @@
       <c r="AJ96" t="inlineStr"/>
       <c r="AK96" t="inlineStr"/>
       <c r="AL96" t="inlineStr"/>
-      <c r="AM96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM96" t="inlineStr"/>
       <c r="AN96" t="inlineStr"/>
       <c r="AO96" t="inlineStr"/>
       <c r="AP96" t="inlineStr"/>
@@ -5128,12 +5043,7 @@
       <c r="AJ99" t="inlineStr"/>
       <c r="AK99" t="inlineStr"/>
       <c r="AL99" t="inlineStr"/>
-      <c r="AM99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM99" t="inlineStr"/>
       <c r="AN99" t="inlineStr"/>
       <c r="AO99" t="inlineStr"/>
       <c r="AP99" t="inlineStr"/>
@@ -5250,12 +5160,7 @@
       <c r="AJ102" t="inlineStr"/>
       <c r="AK102" t="inlineStr"/>
       <c r="AL102" t="inlineStr"/>
-      <c r="AM102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM102" t="inlineStr"/>
       <c r="AN102" t="inlineStr"/>
       <c r="AO102" t="inlineStr"/>
       <c r="AP102" t="inlineStr"/>
@@ -5372,12 +5277,7 @@
       <c r="AJ105" t="inlineStr"/>
       <c r="AK105" t="inlineStr"/>
       <c r="AL105" t="inlineStr"/>
-      <c r="AM105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM105" t="inlineStr"/>
       <c r="AN105" t="inlineStr"/>
       <c r="AO105" t="inlineStr"/>
       <c r="AP105" t="inlineStr"/>
@@ -5494,12 +5394,7 @@
       <c r="AJ108" t="inlineStr"/>
       <c r="AK108" t="inlineStr"/>
       <c r="AL108" t="inlineStr"/>
-      <c r="AM108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM108" t="inlineStr"/>
       <c r="AN108" t="inlineStr"/>
       <c r="AO108" t="inlineStr"/>
       <c r="AP108" t="inlineStr"/>
@@ -5616,12 +5511,7 @@
       <c r="AJ111" t="inlineStr"/>
       <c r="AK111" t="inlineStr"/>
       <c r="AL111" t="inlineStr"/>
-      <c r="AM111" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM111" t="inlineStr"/>
       <c r="AN111" t="inlineStr"/>
       <c r="AO111" t="inlineStr"/>
       <c r="AP111" t="inlineStr"/>
@@ -5738,12 +5628,7 @@
       <c r="AJ114" t="inlineStr"/>
       <c r="AK114" t="inlineStr"/>
       <c r="AL114" t="inlineStr"/>
-      <c r="AM114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM114" t="inlineStr"/>
       <c r="AN114" t="inlineStr"/>
       <c r="AO114" t="inlineStr"/>
       <c r="AP114" t="inlineStr"/>
@@ -5860,12 +5745,7 @@
       <c r="AJ117" t="inlineStr"/>
       <c r="AK117" t="inlineStr"/>
       <c r="AL117" t="inlineStr"/>
-      <c r="AM117" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM117" t="inlineStr"/>
       <c r="AN117" t="inlineStr"/>
       <c r="AO117" t="inlineStr"/>
       <c r="AP117" t="inlineStr"/>
@@ -5982,12 +5862,7 @@
       <c r="AJ120" t="inlineStr"/>
       <c r="AK120" t="inlineStr"/>
       <c r="AL120" t="inlineStr"/>
-      <c r="AM120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM120" t="inlineStr"/>
       <c r="AN120" t="inlineStr"/>
       <c r="AO120" t="inlineStr"/>
       <c r="AP120" t="inlineStr"/>
@@ -6104,12 +5979,7 @@
       <c r="AJ123" t="inlineStr"/>
       <c r="AK123" t="inlineStr"/>
       <c r="AL123" t="inlineStr"/>
-      <c r="AM123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM123" t="inlineStr"/>
       <c r="AN123" t="inlineStr"/>
       <c r="AO123" t="inlineStr"/>
       <c r="AP123" t="inlineStr"/>
@@ -6226,12 +6096,7 @@
       <c r="AJ126" t="inlineStr"/>
       <c r="AK126" t="inlineStr"/>
       <c r="AL126" t="inlineStr"/>
-      <c r="AM126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM126" t="inlineStr"/>
       <c r="AN126" t="inlineStr"/>
       <c r="AO126" t="inlineStr"/>
       <c r="AP126" t="inlineStr"/>
@@ -6348,12 +6213,7 @@
       <c r="AJ129" t="inlineStr"/>
       <c r="AK129" t="inlineStr"/>
       <c r="AL129" t="inlineStr"/>
-      <c r="AM129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM129" t="inlineStr"/>
       <c r="AN129" t="inlineStr"/>
       <c r="AO129" t="inlineStr"/>
       <c r="AP129" t="inlineStr"/>
@@ -6470,12 +6330,7 @@
       <c r="AJ132" t="inlineStr"/>
       <c r="AK132" t="inlineStr"/>
       <c r="AL132" t="inlineStr"/>
-      <c r="AM132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM132" t="inlineStr"/>
       <c r="AN132" t="inlineStr"/>
       <c r="AO132" t="inlineStr"/>
       <c r="AP132" t="inlineStr"/>
@@ -6592,12 +6447,7 @@
       <c r="AJ135" t="inlineStr"/>
       <c r="AK135" t="inlineStr"/>
       <c r="AL135" t="inlineStr"/>
-      <c r="AM135" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM135" t="inlineStr"/>
       <c r="AN135" t="inlineStr"/>
       <c r="AO135" t="inlineStr"/>
       <c r="AP135" t="inlineStr"/>
@@ -6714,12 +6564,7 @@
       <c r="AJ138" t="inlineStr"/>
       <c r="AK138" t="inlineStr"/>
       <c r="AL138" t="inlineStr"/>
-      <c r="AM138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM138" t="inlineStr"/>
       <c r="AN138" t="inlineStr"/>
       <c r="AO138" t="inlineStr"/>
       <c r="AP138" t="inlineStr"/>
@@ -6836,12 +6681,7 @@
       <c r="AJ141" t="inlineStr"/>
       <c r="AK141" t="inlineStr"/>
       <c r="AL141" t="inlineStr"/>
-      <c r="AM141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM141" t="inlineStr"/>
       <c r="AN141" t="inlineStr"/>
       <c r="AO141" t="inlineStr"/>
       <c r="AP141" t="inlineStr"/>
@@ -6958,12 +6798,7 @@
       <c r="AJ144" t="inlineStr"/>
       <c r="AK144" t="inlineStr"/>
       <c r="AL144" t="inlineStr"/>
-      <c r="AM144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM144" t="inlineStr"/>
       <c r="AN144" t="inlineStr"/>
       <c r="AO144" t="inlineStr"/>
       <c r="AP144" t="inlineStr"/>
@@ -7080,12 +6915,7 @@
       <c r="AJ147" t="inlineStr"/>
       <c r="AK147" t="inlineStr"/>
       <c r="AL147" t="inlineStr"/>
-      <c r="AM147" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM147" t="inlineStr"/>
       <c r="AN147" t="inlineStr"/>
       <c r="AO147" t="inlineStr"/>
       <c r="AP147" t="inlineStr"/>
@@ -7202,12 +7032,7 @@
       <c r="AJ150" t="inlineStr"/>
       <c r="AK150" t="inlineStr"/>
       <c r="AL150" t="inlineStr"/>
-      <c r="AM150" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM150" t="inlineStr"/>
       <c r="AN150" t="inlineStr"/>
       <c r="AO150" t="inlineStr"/>
       <c r="AP150" t="inlineStr"/>
@@ -7324,12 +7149,7 @@
       <c r="AJ153" t="inlineStr"/>
       <c r="AK153" t="inlineStr"/>
       <c r="AL153" t="inlineStr"/>
-      <c r="AM153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM153" t="inlineStr"/>
       <c r="AN153" t="inlineStr"/>
       <c r="AO153" t="inlineStr"/>
       <c r="AP153" t="inlineStr"/>
@@ -7446,12 +7266,7 @@
       <c r="AJ156" t="inlineStr"/>
       <c r="AK156" t="inlineStr"/>
       <c r="AL156" t="inlineStr"/>
-      <c r="AM156" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM156" t="inlineStr"/>
       <c r="AN156" t="inlineStr"/>
       <c r="AO156" t="inlineStr"/>
       <c r="AP156" t="inlineStr"/>
@@ -7568,12 +7383,7 @@
       <c r="AJ159" t="inlineStr"/>
       <c r="AK159" t="inlineStr"/>
       <c r="AL159" t="inlineStr"/>
-      <c r="AM159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM159" t="inlineStr"/>
       <c r="AN159" t="inlineStr"/>
       <c r="AO159" t="inlineStr"/>
       <c r="AP159" t="inlineStr"/>
@@ -7690,12 +7500,7 @@
       <c r="AJ162" t="inlineStr"/>
       <c r="AK162" t="inlineStr"/>
       <c r="AL162" t="inlineStr"/>
-      <c r="AM162" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM162" t="inlineStr"/>
       <c r="AN162" t="inlineStr"/>
       <c r="AO162" t="inlineStr"/>
       <c r="AP162" t="inlineStr"/>
@@ -7812,12 +7617,7 @@
       <c r="AJ165" t="inlineStr"/>
       <c r="AK165" t="inlineStr"/>
       <c r="AL165" t="inlineStr"/>
-      <c r="AM165" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM165" t="inlineStr"/>
       <c r="AN165" t="inlineStr"/>
       <c r="AO165" t="inlineStr"/>
       <c r="AP165" t="inlineStr"/>
@@ -7934,12 +7734,7 @@
       <c r="AJ168" t="inlineStr"/>
       <c r="AK168" t="inlineStr"/>
       <c r="AL168" t="inlineStr"/>
-      <c r="AM168" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM168" t="inlineStr"/>
       <c r="AN168" t="inlineStr"/>
       <c r="AO168" t="inlineStr"/>
       <c r="AP168" t="inlineStr"/>
@@ -8056,12 +7851,7 @@
       <c r="AJ171" t="inlineStr"/>
       <c r="AK171" t="inlineStr"/>
       <c r="AL171" t="inlineStr"/>
-      <c r="AM171" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM171" t="inlineStr"/>
       <c r="AN171" t="inlineStr"/>
       <c r="AO171" t="inlineStr"/>
       <c r="AP171" t="inlineStr"/>
@@ -8178,12 +7968,7 @@
       <c r="AJ174" t="inlineStr"/>
       <c r="AK174" t="inlineStr"/>
       <c r="AL174" t="inlineStr"/>
-      <c r="AM174" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM174" t="inlineStr"/>
       <c r="AN174" t="inlineStr"/>
       <c r="AO174" t="inlineStr"/>
       <c r="AP174" t="inlineStr"/>
@@ -8300,12 +8085,7 @@
       <c r="AJ177" t="inlineStr"/>
       <c r="AK177" t="inlineStr"/>
       <c r="AL177" t="inlineStr"/>
-      <c r="AM177" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM177" t="inlineStr"/>
       <c r="AN177" t="inlineStr"/>
       <c r="AO177" t="inlineStr"/>
       <c r="AP177" t="inlineStr"/>
@@ -8422,12 +8202,7 @@
       <c r="AJ180" t="inlineStr"/>
       <c r="AK180" t="inlineStr"/>
       <c r="AL180" t="inlineStr"/>
-      <c r="AM180" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM180" t="inlineStr"/>
       <c r="AN180" t="inlineStr"/>
       <c r="AO180" t="inlineStr"/>
       <c r="AP180" t="inlineStr"/>
@@ -8544,12 +8319,7 @@
       <c r="AJ183" t="inlineStr"/>
       <c r="AK183" t="inlineStr"/>
       <c r="AL183" t="inlineStr"/>
-      <c r="AM183" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM183" t="inlineStr"/>
       <c r="AN183" t="inlineStr"/>
       <c r="AO183" t="inlineStr"/>
       <c r="AP183" t="inlineStr"/>
@@ -8666,12 +8436,7 @@
       <c r="AJ186" t="inlineStr"/>
       <c r="AK186" t="inlineStr"/>
       <c r="AL186" t="inlineStr"/>
-      <c r="AM186" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM186" t="inlineStr"/>
       <c r="AN186" t="inlineStr"/>
       <c r="AO186" t="inlineStr"/>
       <c r="AP186" t="inlineStr"/>
@@ -8788,12 +8553,7 @@
       <c r="AJ189" t="inlineStr"/>
       <c r="AK189" t="inlineStr"/>
       <c r="AL189" t="inlineStr"/>
-      <c r="AM189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM189" t="inlineStr"/>
       <c r="AN189" t="inlineStr"/>
       <c r="AO189" t="inlineStr"/>
       <c r="AP189" t="inlineStr"/>
@@ -8910,12 +8670,7 @@
       <c r="AJ192" t="inlineStr"/>
       <c r="AK192" t="inlineStr"/>
       <c r="AL192" t="inlineStr"/>
-      <c r="AM192" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM192" t="inlineStr"/>
       <c r="AN192" t="inlineStr"/>
       <c r="AO192" t="inlineStr"/>
       <c r="AP192" t="inlineStr"/>
@@ -9032,12 +8787,7 @@
       <c r="AJ195" t="inlineStr"/>
       <c r="AK195" t="inlineStr"/>
       <c r="AL195" t="inlineStr"/>
-      <c r="AM195" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM195" t="inlineStr"/>
       <c r="AN195" t="inlineStr"/>
       <c r="AO195" t="inlineStr"/>
       <c r="AP195" t="inlineStr"/>
@@ -9154,12 +8904,7 @@
       <c r="AJ198" t="inlineStr"/>
       <c r="AK198" t="inlineStr"/>
       <c r="AL198" t="inlineStr"/>
-      <c r="AM198" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM198" t="inlineStr"/>
       <c r="AN198" t="inlineStr"/>
       <c r="AO198" t="inlineStr"/>
       <c r="AP198" t="inlineStr"/>
@@ -9276,12 +9021,7 @@
       <c r="AJ201" t="inlineStr"/>
       <c r="AK201" t="inlineStr"/>
       <c r="AL201" t="inlineStr"/>
-      <c r="AM201" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM201" t="inlineStr"/>
       <c r="AN201" t="inlineStr"/>
       <c r="AO201" t="inlineStr"/>
       <c r="AP201" t="inlineStr"/>
@@ -9398,12 +9138,7 @@
       <c r="AJ204" t="inlineStr"/>
       <c r="AK204" t="inlineStr"/>
       <c r="AL204" t="inlineStr"/>
-      <c r="AM204" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM204" t="inlineStr"/>
       <c r="AN204" t="inlineStr"/>
       <c r="AO204" t="inlineStr"/>
       <c r="AP204" t="inlineStr"/>
@@ -9520,12 +9255,7 @@
       <c r="AJ207" t="inlineStr"/>
       <c r="AK207" t="inlineStr"/>
       <c r="AL207" t="inlineStr"/>
-      <c r="AM207" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM207" t="inlineStr"/>
       <c r="AN207" t="inlineStr"/>
       <c r="AO207" t="inlineStr"/>
       <c r="AP207" t="inlineStr"/>
@@ -9642,12 +9372,7 @@
       <c r="AJ210" t="inlineStr"/>
       <c r="AK210" t="inlineStr"/>
       <c r="AL210" t="inlineStr"/>
-      <c r="AM210" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM210" t="inlineStr"/>
       <c r="AN210" t="inlineStr"/>
       <c r="AO210" t="inlineStr"/>
       <c r="AP210" t="inlineStr"/>
@@ -9764,12 +9489,7 @@
       <c r="AJ213" t="inlineStr"/>
       <c r="AK213" t="inlineStr"/>
       <c r="AL213" t="inlineStr"/>
-      <c r="AM213" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM213" t="inlineStr"/>
       <c r="AN213" t="inlineStr"/>
       <c r="AO213" t="inlineStr"/>
       <c r="AP213" t="inlineStr"/>
@@ -9886,12 +9606,7 @@
       <c r="AJ216" t="inlineStr"/>
       <c r="AK216" t="inlineStr"/>
       <c r="AL216" t="inlineStr"/>
-      <c r="AM216" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM216" t="inlineStr"/>
       <c r="AN216" t="inlineStr"/>
       <c r="AO216" t="inlineStr"/>
       <c r="AP216" t="inlineStr"/>
@@ -10008,12 +9723,7 @@
       <c r="AJ219" t="inlineStr"/>
       <c r="AK219" t="inlineStr"/>
       <c r="AL219" t="inlineStr"/>
-      <c r="AM219" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM219" t="inlineStr"/>
       <c r="AN219" t="inlineStr"/>
       <c r="AO219" t="inlineStr"/>
       <c r="AP219" t="inlineStr"/>
@@ -10130,12 +9840,7 @@
       <c r="AJ222" t="inlineStr"/>
       <c r="AK222" t="inlineStr"/>
       <c r="AL222" t="inlineStr"/>
-      <c r="AM222" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM222" t="inlineStr"/>
       <c r="AN222" t="inlineStr"/>
       <c r="AO222" t="inlineStr"/>
       <c r="AP222" t="inlineStr"/>
@@ -10252,12 +9957,7 @@
       <c r="AJ225" t="inlineStr"/>
       <c r="AK225" t="inlineStr"/>
       <c r="AL225" t="inlineStr"/>
-      <c r="AM225" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM225" t="inlineStr"/>
       <c r="AN225" t="inlineStr"/>
       <c r="AO225" t="inlineStr"/>
       <c r="AP225" t="inlineStr"/>
@@ -10374,12 +10074,7 @@
       <c r="AJ228" t="inlineStr"/>
       <c r="AK228" t="inlineStr"/>
       <c r="AL228" t="inlineStr"/>
-      <c r="AM228" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM228" t="inlineStr"/>
       <c r="AN228" t="inlineStr"/>
       <c r="AO228" t="inlineStr"/>
       <c r="AP228" t="inlineStr"/>
@@ -10496,12 +10191,7 @@
       <c r="AJ231" t="inlineStr"/>
       <c r="AK231" t="inlineStr"/>
       <c r="AL231" t="inlineStr"/>
-      <c r="AM231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM231" t="inlineStr"/>
       <c r="AN231" t="inlineStr"/>
       <c r="AO231" t="inlineStr"/>
       <c r="AP231" t="inlineStr"/>
@@ -10618,12 +10308,7 @@
       <c r="AJ234" t="inlineStr"/>
       <c r="AK234" t="inlineStr"/>
       <c r="AL234" t="inlineStr"/>
-      <c r="AM234" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM234" t="inlineStr"/>
       <c r="AN234" t="inlineStr"/>
       <c r="AO234" t="inlineStr"/>
       <c r="AP234" t="inlineStr"/>
@@ -10740,12 +10425,7 @@
       <c r="AJ237" t="inlineStr"/>
       <c r="AK237" t="inlineStr"/>
       <c r="AL237" t="inlineStr"/>
-      <c r="AM237" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM237" t="inlineStr"/>
       <c r="AN237" t="inlineStr"/>
       <c r="AO237" t="inlineStr"/>
       <c r="AP237" t="inlineStr"/>
@@ -10862,12 +10542,7 @@
       <c r="AJ240" t="inlineStr"/>
       <c r="AK240" t="inlineStr"/>
       <c r="AL240" t="inlineStr"/>
-      <c r="AM240" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM240" t="inlineStr"/>
       <c r="AN240" t="inlineStr"/>
       <c r="AO240" t="inlineStr"/>
       <c r="AP240" t="inlineStr"/>
@@ -10984,12 +10659,7 @@
       <c r="AJ243" t="inlineStr"/>
       <c r="AK243" t="inlineStr"/>
       <c r="AL243" t="inlineStr"/>
-      <c r="AM243" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM243" t="inlineStr"/>
       <c r="AN243" t="inlineStr"/>
       <c r="AO243" t="inlineStr"/>
       <c r="AP243" t="inlineStr"/>
@@ -11106,12 +10776,7 @@
       <c r="AJ246" t="inlineStr"/>
       <c r="AK246" t="inlineStr"/>
       <c r="AL246" t="inlineStr"/>
-      <c r="AM246" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM246" t="inlineStr"/>
       <c r="AN246" t="inlineStr"/>
       <c r="AO246" t="inlineStr"/>
       <c r="AP246" t="inlineStr"/>
@@ -11228,12 +10893,7 @@
       <c r="AJ249" t="inlineStr"/>
       <c r="AK249" t="inlineStr"/>
       <c r="AL249" t="inlineStr"/>
-      <c r="AM249" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM249" t="inlineStr"/>
       <c r="AN249" t="inlineStr"/>
       <c r="AO249" t="inlineStr"/>
       <c r="AP249" t="inlineStr"/>
@@ -11350,12 +11010,7 @@
       <c r="AJ252" t="inlineStr"/>
       <c r="AK252" t="inlineStr"/>
       <c r="AL252" t="inlineStr"/>
-      <c r="AM252" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM252" t="inlineStr"/>
       <c r="AN252" t="inlineStr"/>
       <c r="AO252" t="inlineStr"/>
       <c r="AP252" t="inlineStr"/>
@@ -11472,12 +11127,7 @@
       <c r="AJ255" t="inlineStr"/>
       <c r="AK255" t="inlineStr"/>
       <c r="AL255" t="inlineStr"/>
-      <c r="AM255" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM255" t="inlineStr"/>
       <c r="AN255" t="inlineStr"/>
       <c r="AO255" t="inlineStr"/>
       <c r="AP255" t="inlineStr"/>
@@ -11594,12 +11244,7 @@
       <c r="AJ258" t="inlineStr"/>
       <c r="AK258" t="inlineStr"/>
       <c r="AL258" t="inlineStr"/>
-      <c r="AM258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM258" t="inlineStr"/>
       <c r="AN258" t="inlineStr"/>
       <c r="AO258" t="inlineStr"/>
       <c r="AP258" t="inlineStr"/>
@@ -11716,12 +11361,7 @@
       <c r="AJ261" t="inlineStr"/>
       <c r="AK261" t="inlineStr"/>
       <c r="AL261" t="inlineStr"/>
-      <c r="AM261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM261" t="inlineStr"/>
       <c r="AN261" t="inlineStr"/>
       <c r="AO261" t="inlineStr"/>
       <c r="AP261" t="inlineStr"/>
@@ -11838,12 +11478,7 @@
       <c r="AJ264" t="inlineStr"/>
       <c r="AK264" t="inlineStr"/>
       <c r="AL264" t="inlineStr"/>
-      <c r="AM264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM264" t="inlineStr"/>
       <c r="AN264" t="inlineStr"/>
       <c r="AO264" t="inlineStr"/>
       <c r="AP264" t="inlineStr"/>
@@ -11960,12 +11595,7 @@
       <c r="AJ267" t="inlineStr"/>
       <c r="AK267" t="inlineStr"/>
       <c r="AL267" t="inlineStr"/>
-      <c r="AM267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM267" t="inlineStr"/>
       <c r="AN267" t="inlineStr"/>
       <c r="AO267" t="inlineStr"/>
       <c r="AP267" t="inlineStr"/>
@@ -12082,12 +11712,7 @@
       <c r="AJ270" t="inlineStr"/>
       <c r="AK270" t="inlineStr"/>
       <c r="AL270" t="inlineStr"/>
-      <c r="AM270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM270" t="inlineStr"/>
       <c r="AN270" t="inlineStr"/>
       <c r="AO270" t="inlineStr"/>
       <c r="AP270" t="inlineStr"/>
@@ -12204,12 +11829,7 @@
       <c r="AJ273" t="inlineStr"/>
       <c r="AK273" t="inlineStr"/>
       <c r="AL273" t="inlineStr"/>
-      <c r="AM273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM273" t="inlineStr"/>
       <c r="AN273" t="inlineStr"/>
       <c r="AO273" t="inlineStr"/>
       <c r="AP273" t="inlineStr"/>
@@ -12326,12 +11946,7 @@
       <c r="AJ276" t="inlineStr"/>
       <c r="AK276" t="inlineStr"/>
       <c r="AL276" t="inlineStr"/>
-      <c r="AM276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM276" t="inlineStr"/>
       <c r="AN276" t="inlineStr"/>
       <c r="AO276" t="inlineStr"/>
       <c r="AP276" t="inlineStr"/>
@@ -12448,12 +12063,7 @@
       <c r="AJ279" t="inlineStr"/>
       <c r="AK279" t="inlineStr"/>
       <c r="AL279" t="inlineStr"/>
-      <c r="AM279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM279" t="inlineStr"/>
       <c r="AN279" t="inlineStr"/>
       <c r="AO279" t="inlineStr"/>
       <c r="AP279" t="inlineStr"/>
@@ -12570,12 +12180,7 @@
       <c r="AJ282" t="inlineStr"/>
       <c r="AK282" t="inlineStr"/>
       <c r="AL282" t="inlineStr"/>
-      <c r="AM282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM282" t="inlineStr"/>
       <c r="AN282" t="inlineStr"/>
       <c r="AO282" t="inlineStr"/>
       <c r="AP282" t="inlineStr"/>
@@ -12692,12 +12297,7 @@
       <c r="AJ285" t="inlineStr"/>
       <c r="AK285" t="inlineStr"/>
       <c r="AL285" t="inlineStr"/>
-      <c r="AM285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM285" t="inlineStr"/>
       <c r="AN285" t="inlineStr"/>
       <c r="AO285" t="inlineStr"/>
       <c r="AP285" t="inlineStr"/>
@@ -12814,12 +12414,7 @@
       <c r="AJ288" t="inlineStr"/>
       <c r="AK288" t="inlineStr"/>
       <c r="AL288" t="inlineStr"/>
-      <c r="AM288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM288" t="inlineStr"/>
       <c r="AN288" t="inlineStr"/>
       <c r="AO288" t="inlineStr"/>
       <c r="AP288" t="inlineStr"/>
@@ -12936,12 +12531,7 @@
       <c r="AJ291" t="inlineStr"/>
       <c r="AK291" t="inlineStr"/>
       <c r="AL291" t="inlineStr"/>
-      <c r="AM291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM291" t="inlineStr"/>
       <c r="AN291" t="inlineStr"/>
       <c r="AO291" t="inlineStr"/>
       <c r="AP291" t="inlineStr"/>
@@ -13058,12 +12648,7 @@
       <c r="AJ294" t="inlineStr"/>
       <c r="AK294" t="inlineStr"/>
       <c r="AL294" t="inlineStr"/>
-      <c r="AM294" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM294" t="inlineStr"/>
       <c r="AN294" t="inlineStr"/>
       <c r="AO294" t="inlineStr"/>
       <c r="AP294" t="inlineStr"/>
@@ -13180,12 +12765,7 @@
       <c r="AJ297" t="inlineStr"/>
       <c r="AK297" t="inlineStr"/>
       <c r="AL297" t="inlineStr"/>
-      <c r="AM297" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM297" t="inlineStr"/>
       <c r="AN297" t="inlineStr"/>
       <c r="AO297" t="inlineStr"/>
       <c r="AP297" t="inlineStr"/>
@@ -13302,12 +12882,7 @@
       <c r="AJ300" t="inlineStr"/>
       <c r="AK300" t="inlineStr"/>
       <c r="AL300" t="inlineStr"/>
-      <c r="AM300" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM300" t="inlineStr"/>
       <c r="AN300" t="inlineStr"/>
       <c r="AO300" t="inlineStr"/>
       <c r="AP300" t="inlineStr"/>

</xml_diff>

<commit_message>
add noice to delay calculation (!! not finish !!!)
</commit_message>
<xml_diff>
--- a/debug.xlsx
+++ b/debug.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="State" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1293,26 +1293,10 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 18];
-rreg:[31, 37, 40, 22, 5, 24];
-rreg:[31, 37, 40, 22, 5, 39];
-rreg:[31, 37, 40, 22, 5, 45];
-</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 8, 24];
-rreg:[31, 37, 40, 22, 8, 47];
-rreg:[31, 37, 40, 22, 8, 39];
-rreg:[31, 37, 40, 22, 8, 21];
-</t>
-        </is>
-      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1340,7 +1324,13 @@
 </t>
         </is>
       </c>
-      <c r="X15" t="inlineStr"/>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
@@ -1457,18 +1447,29 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8];
+</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 24, 8];
-</t>
-        </is>
-      </c>
+      <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
@@ -1483,14 +1484,7 @@
       <c r="AL18" t="inlineStr"/>
       <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
-      <c r="AO18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 39, 8];
-rreg:[31, 37, 40, 22, 5, 39, 20];
-rreg:[31, 37, 40, 22, 5, 39, 42];
-</t>
-        </is>
-      </c>
+      <c r="AO18" t="inlineStr"/>
       <c r="AP18" t="inlineStr"/>
       <c r="AQ18" t="inlineStr"/>
       <c r="AR18" t="inlineStr"/>
@@ -1498,20 +1492,15 @@
       <c r="AT18" t="inlineStr"/>
       <c r="AU18" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 2];
-rreg:[31, 37, 40, 22, 5, 45, 9];
-rreg:[31, 37, 40, 22, 5, 45, 18];
-rreg:[31, 37, 40, 22, 5, 45, 20];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 2];
+rreg:[31, 37, 40, 22, 18, 45, 5];
+rreg:[31, 37, 40, 22, 18, 45, 9];
+rreg:[31, 37, 40, 22, 18, 45, 20];
 </t>
         </is>
       </c>
       <c r="AV18" t="inlineStr"/>
-      <c r="AW18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 8, 47, 4];
-</t>
-        </is>
-      </c>
+      <c r="AW18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1589,28 +1578,22 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 2, 9];
-rreg:[31, 37, 40, 22, 5, 45, 2, 20];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 2, 9];
+rreg:[31, 37, 40, 22, 18, 45, 2, 20];
 </t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 8, 47, 4, 9];
-rreg:[31, 37, 40, 22, 8, 47, 4, 10];
-</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 9, 2];
-rreg:[31, 37, 40, 22, 5, 45, 9, 4];
-rreg:[31, 37, 40, 22, 5, 45, 9, 27];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 9, 2];
+rreg:[31, 37, 40, 22, 18, 45, 9, 4];
+rreg:[31, 37, 40, 22, 18, 45, 9, 27];
 </t>
         </is>
       </c>
@@ -1622,19 +1605,35 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 2];
-rreg:[31, 37, 40, 22, 5, 45, 20, 27];
-rreg:[31, 37, 40, 22, 5, 45, 20, 38];
-rreg:[31, 37, 40, 22, 5, 45, 20, 39];
-</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 2];
+rreg:[31, 37, 40, 22, 18, 45, 20, 27];
+rreg:[31, 37, 40, 22, 18, 45, 20, 38];
+rreg:[31, 37, 40, 22, 18, 45, 20, 39];
+</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8];
+</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
@@ -1654,17 +1653,15 @@
       <c r="AO21" t="inlineStr"/>
       <c r="AP21" t="inlineStr"/>
       <c r="AQ21" t="inlineStr"/>
-      <c r="AR21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 39, 42, 33];
-rreg:[31, 37, 40, 22, 5, 39, 42, 43];
-rreg:[31, 37, 40, 22, 5, 39, 42, 43];
-</t>
-        </is>
-      </c>
+      <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="inlineStr"/>
       <c r="AT21" t="inlineStr"/>
-      <c r="AU21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV21" t="inlineStr"/>
       <c r="AW21" t="inlineStr"/>
     </row>
@@ -1744,18 +1741,19 @@
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 9, 4, 47];
+rreg:[31, 37, 40, 22, 18, 45, 9, 4, 10];
+</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 8, 47, 4, 10, 1];
-</t>
-        </is>
-      </c>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
@@ -1763,19 +1761,35 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8];
+</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 9, 27, 1];
-rreg:[31, 37, 40, 22, 5, 45, 9, 27, 20];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 9, 27, 1];
+rreg:[31, 37, 40, 22, 18, 45, 9, 27, 20];
 </t>
         </is>
       </c>
@@ -1784,36 +1798,37 @@
       <c r="AF24" t="inlineStr"/>
       <c r="AG24" t="inlineStr"/>
       <c r="AH24" t="inlineStr"/>
-      <c r="AI24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AI24" t="inlineStr"/>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
       <c r="AL24" t="inlineStr"/>
       <c r="AM24" t="inlineStr"/>
       <c r="AN24" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 12];
-rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15];
-</t>
-        </is>
-      </c>
-      <c r="AO24" t="inlineStr"/>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 38, 12];
+rreg:[31, 37, 40, 22, 18, 45, 20, 38, 15];
+</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5];
+rreg:[31, 37, 40, 22, 18, 45, 20, 39, 8];
+rreg:[31, 37, 40, 22, 18, 45, 20, 39, 42];
+</t>
+        </is>
+      </c>
       <c r="AP24" t="inlineStr"/>
       <c r="AQ24" t="inlineStr"/>
       <c r="AR24" t="inlineStr"/>
-      <c r="AS24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 39, 42, 43, 13];
-rreg:[31, 37, 40, 22, 5, 39, 42, 43, 33];
-</t>
-        </is>
-      </c>
+      <c r="AS24" t="inlineStr"/>
       <c r="AT24" t="inlineStr"/>
-      <c r="AU24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV24" t="inlineStr"/>
       <c r="AW24" t="inlineStr"/>
     </row>
@@ -1892,48 +1907,69 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 9, 27, 1, 10];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 9, 27, 1, 10];
 </t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 9, 4, 10, 1];
+</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6];
-rreg:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26];
-</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33];
-</t>
-        </is>
-      </c>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6];
+rreg:[31, 37, 40, 22, 18, 45, 20, 38, 12, 26];
+</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15, 26];
-rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 38, 15, 26];
+rreg:[31, 37, 40, 22, 18, 45, 20, 38, 15, 25];
 </t>
         </is>
       </c>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8];
+</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="inlineStr"/>
@@ -1944,31 +1980,43 @@
       <c r="AF27" t="inlineStr"/>
       <c r="AG27" t="inlineStr"/>
       <c r="AH27" t="inlineStr"/>
-      <c r="AI27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AI27" t="inlineStr"/>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
       <c r="AL27" t="inlineStr"/>
       <c r="AM27" t="inlineStr"/>
       <c r="AN27" t="inlineStr"/>
-      <c r="AO27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 8];
+</t>
+        </is>
+      </c>
       <c r="AP27" t="inlineStr"/>
       <c r="AQ27" t="inlineStr"/>
       <c r="AR27" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 42, 33];
+rreg:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43];
+rreg:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43];
 </t>
         </is>
       </c>
       <c r="AS27" t="inlineStr"/>
       <c r="AT27" t="inlineStr"/>
-      <c r="AU27" t="inlineStr"/>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV27" t="inlineStr"/>
-      <c r="AW27" t="inlineStr"/>
+      <c r="AW27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8];
+</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2047,15 +2095,27 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
 </t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 47];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
@@ -2065,23 +2125,34 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6];
-rreg:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 16];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 38, 15, 25, 6];
+rreg:[31, 37, 40, 22, 18, 45, 20, 38, 15, 25, 16];
 </t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 38, 12, 26, 15];
 </t>
         </is>
       </c>
@@ -2093,7 +2164,7 @@
       <c r="AH30" t="inlineStr"/>
       <c r="AI30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 33, 23];
 </t>
         </is>
       </c>
@@ -2104,9 +2175,7 @@
       <c r="AN30" t="inlineStr"/>
       <c r="AO30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 8];
 </t>
         </is>
       </c>
@@ -2115,15 +2184,25 @@
       <c r="AR30" t="inlineStr"/>
       <c r="AS30" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
-rrep:[31, 37, 40, 22, 5, 39, 42, 43, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43, 13];
+rreg:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43, 33];
 </t>
         </is>
       </c>
       <c r="AT30" t="inlineStr"/>
-      <c r="AU30" t="inlineStr"/>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV30" t="inlineStr"/>
-      <c r="AW30" t="inlineStr"/>
+      <c r="AW30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8];
+</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2204,24 +2283,22 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
 </t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 15, 25, 6, 23];
 </t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 24, 8, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 39, 8, 39, 42, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 47];
+rreg:[31, 37, 40, 22, 21, 8, 39];
 </t>
         </is>
       </c>
@@ -2230,13 +2307,13 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
 </t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 43, 13, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43, 13, 33];
 </t>
         </is>
       </c>
@@ -2244,24 +2321,27 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 16, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 15, 25, 16, 23];
 </t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 39, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 2, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 9, 27, 20, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
       <c r="AA33" t="inlineStr"/>
@@ -2272,21 +2352,41 @@
       <c r="AF33" t="inlineStr"/>
       <c r="AG33" t="inlineStr"/>
       <c r="AH33" t="inlineStr"/>
-      <c r="AI33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AJ33" t="inlineStr"/>
       <c r="AK33" t="inlineStr"/>
       <c r="AL33" t="inlineStr"/>
       <c r="AM33" t="inlineStr"/>
       <c r="AN33" t="inlineStr"/>
-      <c r="AO33" t="inlineStr"/>
+      <c r="AO33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 8];
+</t>
+        </is>
+      </c>
       <c r="AP33" t="inlineStr"/>
       <c r="AQ33" t="inlineStr"/>
-      <c r="AR33" t="inlineStr"/>
+      <c r="AR33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AS33" t="inlineStr"/>
       <c r="AT33" t="inlineStr"/>
       <c r="AU33" t="inlineStr"/>
       <c r="AV33" t="inlineStr"/>
-      <c r="AW33" t="inlineStr"/>
+      <c r="AW33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8];
+</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2362,20 +2462,25 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 2, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 9, 2, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 20, 2, 20, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 47];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
@@ -2387,81 +2492,70 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 18, 5, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 21, 18, 5, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 18, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
 </t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 8, 21, 8, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 18, 21, 8, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
 </t>
         </is>
       </c>
       <c r="Y36" t="inlineStr"/>
-      <c r="Z36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 24, 8, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 8, 24, 8, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="Z36" t="inlineStr"/>
       <c r="AA36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 15, 25, 6, 23];
 </t>
         </is>
       </c>
       <c r="AB36" t="inlineStr"/>
-      <c r="AC36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 9, 27, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 20, 27, 20, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AC36" t="inlineStr"/>
       <c r="AD36" t="inlineStr"/>
       <c r="AE36" t="inlineStr"/>
       <c r="AF36" t="inlineStr"/>
       <c r="AG36" t="inlineStr"/>
       <c r="AH36" t="inlineStr"/>
-      <c r="AI36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43, 13, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AJ36" t="inlineStr"/>
       <c r="AK36" t="inlineStr"/>
       <c r="AL36" t="inlineStr"/>
       <c r="AM36" t="inlineStr"/>
       <c r="AN36" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 6, 23];
-</t>
-        </is>
-      </c>
-      <c r="AO36" t="inlineStr"/>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="AO36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 8];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP36" t="inlineStr"/>
       <c r="AQ36" t="inlineStr"/>
       <c r="AR36" t="inlineStr"/>
-      <c r="AS36" t="inlineStr"/>
+      <c r="AS36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AT36" t="inlineStr"/>
-      <c r="AU36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AU36" t="inlineStr"/>
       <c r="AV36" t="inlineStr"/>
       <c r="AW36" t="inlineStr"/>
     </row>
@@ -2542,50 +2636,72 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 9, 2, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 2, 9, 2, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 47];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 39, 42, 43, 13, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 25, 6, 23];
-rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15, 25, 6, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 15, 25, 6, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 26, 15, 25, 6, 23];
 </t>
         </is>
       </c>
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 18, 45, 2, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 27, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr"/>
       <c r="AC39" t="inlineStr"/>
       <c r="AD39" t="inlineStr"/>
-      <c r="AE39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 18, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AE39" t="inlineStr"/>
       <c r="AF39" t="inlineStr"/>
       <c r="AG39" t="inlineStr"/>
       <c r="AH39" t="inlineStr"/>
@@ -2596,12 +2712,7 @@
       <c r="AM39" t="inlineStr"/>
       <c r="AN39" t="inlineStr"/>
       <c r="AO39" t="inlineStr"/>
-      <c r="AP39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AP39" t="inlineStr"/>
       <c r="AQ39" t="inlineStr"/>
       <c r="AR39" t="inlineStr"/>
       <c r="AS39" t="inlineStr"/>
@@ -2684,51 +2795,74 @@
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 2, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 2, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 2, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
-rrep:[31, 37, 40, 22, 5, 45, 9, 4, 9, 2, 20, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 47];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 3, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
-      <c r="T42" t="inlineStr"/>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr">
         <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 45, 20, 38, 12, 26, 15, 25, 6, 23];
-rrep:[31, 37, 40, 22, 5, 45, 20, 38, 15, 26, 15, 25, 6, 23];
-</t>
-        </is>
-      </c>
-      <c r="AC42" t="inlineStr"/>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 26, 15, 25, 6, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 38, 15, 26, 15, 25, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 27, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 27, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AD42" t="inlineStr"/>
       <c r="AE42" t="inlineStr"/>
       <c r="AF42" t="inlineStr"/>
@@ -2738,13 +2872,7 @@
       <c r="AJ42" t="inlineStr"/>
       <c r="AK42" t="inlineStr"/>
       <c r="AL42" t="inlineStr"/>
-      <c r="AM42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep:[31, 44, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM42" t="inlineStr"/>
       <c r="AN42" t="inlineStr"/>
       <c r="AO42" t="inlineStr"/>
       <c r="AP42" t="inlineStr"/>
@@ -2752,7 +2880,12 @@
       <c r="AR42" t="inlineStr"/>
       <c r="AS42" t="inlineStr"/>
       <c r="AT42" t="inlineStr"/>
-      <c r="AU42" t="inlineStr"/>
+      <c r="AU42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AV42" t="inlineStr"/>
       <c r="AW42" t="inlineStr"/>
     </row>
@@ -2833,11 +2966,28 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 2, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 18, 45, 2, 9, 2, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
@@ -2846,34 +2996,34 @@
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 21, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr"/>
       <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y45" t="inlineStr"/>
       <c r="Z45" t="inlineStr"/>
       <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr"/>
       <c r="AC45" t="inlineStr"/>
-      <c r="AD45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 46, 3, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 11, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 3, 41, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 11, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AD45" t="inlineStr"/>
       <c r="AE45" t="inlineStr"/>
       <c r="AF45" t="inlineStr"/>
-      <c r="AG45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AG45" t="inlineStr"/>
       <c r="AH45" t="inlineStr"/>
       <c r="AI45" t="inlineStr"/>
       <c r="AJ45" t="inlineStr"/>
@@ -2883,39 +3033,13 @@
       <c r="AN45" t="inlineStr"/>
       <c r="AO45" t="inlineStr"/>
       <c r="AP45" t="inlineStr"/>
-      <c r="AQ45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 11, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 3, 28, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 11, 30, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AQ45" t="inlineStr"/>
       <c r="AR45" t="inlineStr"/>
       <c r="AS45" t="inlineStr"/>
-      <c r="AT45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 44, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep:[31, 34, 44, 37, 40, 22, 5, 39, 42, 33, 23];
-rrep:[31, 37, 44, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AT45" t="inlineStr"/>
       <c r="AU45" t="inlineStr"/>
-      <c r="AV45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
-      <c r="AW45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 37, 40, 22, 8, 47, 4, 9, 2, 20, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AV45" t="inlineStr"/>
+      <c r="AW45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2954,7 +3078,11 @@
       <c r="AD46" t="inlineStr"/>
       <c r="AE46" t="inlineStr"/>
       <c r="AF46" t="inlineStr"/>
-      <c r="AG46" t="inlineStr"/>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>-1;</t>
+        </is>
+      </c>
       <c r="AH46" t="inlineStr"/>
       <c r="AI46" t="inlineStr"/>
       <c r="AJ46" t="inlineStr"/>
@@ -2988,23 +3116,23 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 46, 3, 41, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 46, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 3, 28, 7, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
@@ -3014,46 +3142,50 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr"/>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 18, 21, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="Y48" t="inlineStr"/>
       <c r="Z48" t="inlineStr"/>
       <c r="AA48" t="inlineStr"/>
       <c r="AB48" t="inlineStr"/>
       <c r="AC48" t="inlineStr"/>
       <c r="AD48" t="inlineStr"/>
-      <c r="AE48" t="inlineStr"/>
-      <c r="AF48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 46, 11, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 3, 28, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 3, 41, 30, 28, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 37, 40, 22, 18, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr"/>
       <c r="AG48" t="inlineStr"/>
       <c r="AH48" t="inlineStr"/>
       <c r="AI48" t="inlineStr"/>
-      <c r="AJ48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 46, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 44, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AJ48" t="inlineStr"/>
       <c r="AK48" t="inlineStr"/>
       <c r="AL48" t="inlineStr"/>
-      <c r="AM48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AM48" t="inlineStr"/>
       <c r="AN48" t="inlineStr"/>
       <c r="AO48" t="inlineStr"/>
       <c r="AP48" t="inlineStr"/>
@@ -3102,7 +3234,11 @@
       <c r="AD49" t="inlineStr"/>
       <c r="AE49" t="inlineStr"/>
       <c r="AF49" t="inlineStr"/>
-      <c r="AG49" t="inlineStr"/>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>-1;</t>
+        </is>
+      </c>
       <c r="AH49" t="inlineStr"/>
       <c r="AI49" t="inlineStr"/>
       <c r="AJ49" t="inlineStr"/>
@@ -3138,24 +3274,53 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 3, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 3, 41, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr"/>
-      <c r="T51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr"/>
       <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y51" t="inlineStr"/>
       <c r="Z51" t="inlineStr"/>
       <c r="AA51" t="inlineStr"/>
@@ -3165,13 +3330,7 @@
       <c r="AE51" t="inlineStr"/>
       <c r="AF51" t="inlineStr"/>
       <c r="AG51" t="inlineStr"/>
-      <c r="AH51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rrep:[31, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-rrep:[31, 34, 32, 34, 46, 11, 29, 18, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AH51" t="inlineStr"/>
       <c r="AI51" t="inlineStr"/>
       <c r="AJ51" t="inlineStr"/>
       <c r="AK51" t="inlineStr"/>
@@ -3181,7 +3340,7 @@
       <c r="AO51" t="inlineStr"/>
       <c r="AP51" t="inlineStr">
         <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
 </t>
         </is>
       </c>
@@ -3230,7 +3389,11 @@
       <c r="AD52" t="inlineStr"/>
       <c r="AE52" t="inlineStr"/>
       <c r="AF52" t="inlineStr"/>
-      <c r="AG52" t="inlineStr"/>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>-1;</t>
+        </is>
+      </c>
       <c r="AH52" t="inlineStr"/>
       <c r="AI52" t="inlineStr"/>
       <c r="AJ52" t="inlineStr"/>
@@ -3266,10 +3429,21 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
@@ -3279,13 +3453,19 @@
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="inlineStr"/>
-      <c r="T54" t="inlineStr"/>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr"/>
       <c r="W54" t="inlineStr"/>
       <c r="X54" t="inlineStr">
         <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
 </t>
         </is>
       </c>
@@ -3294,7 +3474,16 @@
       <c r="AA54" t="inlineStr"/>
       <c r="AB54" t="inlineStr"/>
       <c r="AC54" t="inlineStr"/>
-      <c r="AD54" t="inlineStr"/>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 46, 3, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 7, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 11, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 3, 41, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 11, 30, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AE54" t="inlineStr"/>
       <c r="AF54" t="inlineStr"/>
       <c r="AG54" t="inlineStr"/>
@@ -3303,16 +3492,36 @@
       <c r="AJ54" t="inlineStr"/>
       <c r="AK54" t="inlineStr"/>
       <c r="AL54" t="inlineStr"/>
-      <c r="AM54" t="inlineStr"/>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 44, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AN54" t="inlineStr"/>
       <c r="AO54" t="inlineStr"/>
       <c r="AP54" t="inlineStr"/>
-      <c r="AQ54" t="inlineStr"/>
+      <c r="AQ54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 46, 3, 41, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 11, 41, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 3, 28, 41, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 11, 30, 41, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AR54" t="inlineStr"/>
       <c r="AS54" t="inlineStr"/>
       <c r="AT54" t="inlineStr"/>
       <c r="AU54" t="inlineStr"/>
-      <c r="AV54" t="inlineStr"/>
+      <c r="AV54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 34, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AW54" t="inlineStr"/>
     </row>
     <row r="55">
@@ -3352,7 +3561,11 @@
       <c r="AD55" t="inlineStr"/>
       <c r="AE55" t="inlineStr"/>
       <c r="AF55" t="inlineStr"/>
-      <c r="AG55" t="inlineStr"/>
+      <c r="AG55" t="inlineStr">
+        <is>
+          <t>-1;</t>
+        </is>
+      </c>
       <c r="AH55" t="inlineStr"/>
       <c r="AI55" t="inlineStr"/>
       <c r="AJ55" t="inlineStr"/>
@@ -3386,17 +3599,34 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 46, 3, 41, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
 </t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 46, 7, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 3, 28, 7, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
@@ -3406,11 +3636,22 @@
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="inlineStr"/>
-      <c r="T57" t="inlineStr"/>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U57" t="inlineStr"/>
       <c r="V57" t="inlineStr"/>
       <c r="W57" t="inlineStr"/>
-      <c r="X57" t="inlineStr"/>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y57" t="inlineStr"/>
       <c r="Z57" t="inlineStr"/>
       <c r="AA57" t="inlineStr"/>
@@ -3418,11 +3659,31 @@
       <c r="AC57" t="inlineStr"/>
       <c r="AD57" t="inlineStr"/>
       <c r="AE57" t="inlineStr"/>
-      <c r="AF57" t="inlineStr"/>
-      <c r="AG57" t="inlineStr"/>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 46, 11, 30, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 3, 28, 30, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 3, 41, 30, 28, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AH57" t="inlineStr"/>
       <c r="AI57" t="inlineStr"/>
-      <c r="AJ57" t="inlineStr"/>
+      <c r="AJ57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 34, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 32, 34, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 46, 34, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 44, 34, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AK57" t="inlineStr"/>
       <c r="AL57" t="inlineStr"/>
       <c r="AM57" t="inlineStr"/>
@@ -3432,7 +3693,14 @@
       <c r="AQ57" t="inlineStr"/>
       <c r="AR57" t="inlineStr"/>
       <c r="AS57" t="inlineStr"/>
-      <c r="AT57" t="inlineStr"/>
+      <c r="AT57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 44, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 34, 44, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 37, 44, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AU57" t="inlineStr"/>
       <c r="AV57" t="inlineStr"/>
       <c r="AW57" t="inlineStr"/>
@@ -3510,10 +3778,21 @@
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
@@ -3523,11 +3802,22 @@
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
-      <c r="T60" t="inlineStr"/>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr"/>
       <c r="W60" t="inlineStr"/>
-      <c r="X60" t="inlineStr"/>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y60" t="inlineStr"/>
       <c r="Z60" t="inlineStr"/>
       <c r="AA60" t="inlineStr"/>
@@ -3537,19 +3827,25 @@
       <c r="AE60" t="inlineStr"/>
       <c r="AF60" t="inlineStr"/>
       <c r="AG60" t="inlineStr"/>
-      <c r="AH60" t="inlineStr"/>
+      <c r="AH60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 32, 34, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+rrep:[31, 34, 32, 34, 46, 11, 29, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AI60" t="inlineStr"/>
       <c r="AJ60" t="inlineStr"/>
       <c r="AK60" t="inlineStr"/>
       <c r="AL60" t="inlineStr"/>
-      <c r="AM60" t="inlineStr"/>
+      <c r="AM60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AN60" t="inlineStr"/>
-      <c r="AO60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AO60" t="inlineStr"/>
       <c r="AP60" t="inlineStr"/>
       <c r="AQ60" t="inlineStr"/>
       <c r="AR60" t="inlineStr"/>
@@ -3632,10 +3928,21 @@
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
@@ -3645,11 +3952,22 @@
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr"/>
-      <c r="T63" t="inlineStr"/>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U63" t="inlineStr"/>
       <c r="V63" t="inlineStr"/>
       <c r="W63" t="inlineStr"/>
-      <c r="X63" t="inlineStr"/>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y63" t="inlineStr"/>
       <c r="Z63" t="inlineStr"/>
       <c r="AA63" t="inlineStr"/>
@@ -3667,14 +3985,14 @@
       <c r="AM63" t="inlineStr"/>
       <c r="AN63" t="inlineStr"/>
       <c r="AO63" t="inlineStr"/>
-      <c r="AP63" t="inlineStr"/>
+      <c r="AP63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AQ63" t="inlineStr"/>
-      <c r="AR63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AR63" t="inlineStr"/>
       <c r="AS63" t="inlineStr"/>
       <c r="AT63" t="inlineStr"/>
       <c r="AU63" t="inlineStr"/>
@@ -3754,10 +4072,21 @@
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+rreg:[31, 37, 40, 22, 21, 8, 39];
+</t>
+        </is>
+      </c>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
@@ -3767,11 +4096,23 @@
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr"/>
-      <c r="T66" t="inlineStr"/>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U66" t="inlineStr"/>
       <c r="V66" t="inlineStr"/>
       <c r="W66" t="inlineStr"/>
-      <c r="X66" t="inlineStr"/>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="Y66" t="inlineStr"/>
       <c r="Z66" t="inlineStr"/>
       <c r="AA66" t="inlineStr"/>
@@ -3782,12 +4123,7 @@
       <c r="AF66" t="inlineStr"/>
       <c r="AG66" t="inlineStr"/>
       <c r="AH66" t="inlineStr"/>
-      <c r="AI66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">data:[31, 37, 40, 22, 5, 39, 42, 33, 23];
-</t>
-        </is>
-      </c>
+      <c r="AI66" t="inlineStr"/>
       <c r="AJ66" t="inlineStr"/>
       <c r="AK66" t="inlineStr"/>
       <c r="AL66" t="inlineStr"/>
@@ -3876,10 +4212,20 @@
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
@@ -3889,11 +4235,23 @@
       <c r="Q69" t="inlineStr"/>
       <c r="R69" t="inlineStr"/>
       <c r="S69" t="inlineStr"/>
-      <c r="T69" t="inlineStr"/>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr"/>
       <c r="W69" t="inlineStr"/>
-      <c r="X69" t="inlineStr"/>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y69" t="inlineStr"/>
       <c r="Z69" t="inlineStr"/>
       <c r="AA69" t="inlineStr"/>
@@ -3910,7 +4268,14 @@
       <c r="AL69" t="inlineStr"/>
       <c r="AM69" t="inlineStr"/>
       <c r="AN69" t="inlineStr"/>
-      <c r="AO69" t="inlineStr"/>
+      <c r="AO69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20];
+rreg:[31, 37, 40, 22, 21, 8, 39, 42];
+</t>
+        </is>
+      </c>
       <c r="AP69" t="inlineStr"/>
       <c r="AQ69" t="inlineStr"/>
       <c r="AR69" t="inlineStr"/>
@@ -3993,10 +4358,20 @@
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
@@ -4006,11 +4381,30 @@
       <c r="Q72" t="inlineStr"/>
       <c r="R72" t="inlineStr"/>
       <c r="S72" t="inlineStr"/>
-      <c r="T72" t="inlineStr"/>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U72" t="inlineStr"/>
-      <c r="V72" t="inlineStr"/>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 2];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 27];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38];
+</t>
+        </is>
+      </c>
       <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y72" t="inlineStr"/>
       <c r="Z72" t="inlineStr"/>
       <c r="AA72" t="inlineStr"/>
@@ -4027,13 +4421,30 @@
       <c r="AL72" t="inlineStr"/>
       <c r="AM72" t="inlineStr"/>
       <c r="AN72" t="inlineStr"/>
-      <c r="AO72" t="inlineStr"/>
+      <c r="AO72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+</t>
+        </is>
+      </c>
       <c r="AP72" t="inlineStr"/>
       <c r="AQ72" t="inlineStr"/>
-      <c r="AR72" t="inlineStr"/>
+      <c r="AR72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 42, 33];
+rreg:[31, 37, 40, 22, 21, 8, 39, 42, 43];
+rreg:[31, 37, 40, 22, 21, 8, 39, 42, 43];
+</t>
+        </is>
+      </c>
       <c r="AS72" t="inlineStr"/>
       <c r="AT72" t="inlineStr"/>
-      <c r="AU72" t="inlineStr"/>
+      <c r="AU72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AV72" t="inlineStr"/>
       <c r="AW72" t="inlineStr"/>
     </row>
@@ -4107,13 +4518,29 @@
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 2, 45];
+</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr"/>
@@ -4123,34 +4550,86 @@
       <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="inlineStr"/>
-      <c r="T75" t="inlineStr"/>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U75" t="inlineStr"/>
-      <c r="V75" t="inlineStr"/>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="W75" t="inlineStr"/>
-      <c r="X75" t="inlineStr"/>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y75" t="inlineStr"/>
       <c r="Z75" t="inlineStr"/>
       <c r="AA75" t="inlineStr"/>
       <c r="AB75" t="inlineStr"/>
-      <c r="AC75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 27, 1];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 27, 9];
+</t>
+        </is>
+      </c>
       <c r="AD75" t="inlineStr"/>
       <c r="AE75" t="inlineStr"/>
       <c r="AF75" t="inlineStr"/>
       <c r="AG75" t="inlineStr"/>
       <c r="AH75" t="inlineStr"/>
-      <c r="AI75" t="inlineStr"/>
+      <c r="AI75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AJ75" t="inlineStr"/>
       <c r="AK75" t="inlineStr"/>
       <c r="AL75" t="inlineStr"/>
       <c r="AM75" t="inlineStr"/>
-      <c r="AN75" t="inlineStr"/>
-      <c r="AO75" t="inlineStr"/>
+      <c r="AN75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15];
+</t>
+        </is>
+      </c>
+      <c r="AO75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+</t>
+        </is>
+      </c>
       <c r="AP75" t="inlineStr"/>
       <c r="AQ75" t="inlineStr"/>
       <c r="AR75" t="inlineStr"/>
-      <c r="AS75" t="inlineStr"/>
+      <c r="AS75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 42, 43, 13];
+rreg:[31, 37, 40, 22, 21, 8, 39, 42, 43, 33];
+</t>
+        </is>
+      </c>
       <c r="AT75" t="inlineStr"/>
-      <c r="AU75" t="inlineStr"/>
+      <c r="AU75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 2];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 9];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18];
+</t>
+        </is>
+      </c>
       <c r="AV75" t="inlineStr"/>
       <c r="AW75" t="inlineStr"/>
     </row>
@@ -4227,24 +4706,71 @@
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9, 4];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9, 45];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9, 27];
+</t>
+        </is>
+      </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 6];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 26];
+</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 42, 43, 13, 33];
+</t>
+        </is>
+      </c>
       <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 26];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 25];
+</t>
+        </is>
+      </c>
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr"/>
-      <c r="T78" t="inlineStr"/>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 5];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29];
+</t>
+        </is>
+      </c>
       <c r="U78" t="inlineStr"/>
       <c r="V78" t="inlineStr"/>
       <c r="W78" t="inlineStr"/>
-      <c r="X78" t="inlineStr"/>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y78" t="inlineStr"/>
       <c r="Z78" t="inlineStr"/>
       <c r="AA78" t="inlineStr"/>
@@ -4255,19 +4781,44 @@
       <c r="AF78" t="inlineStr"/>
       <c r="AG78" t="inlineStr"/>
       <c r="AH78" t="inlineStr"/>
-      <c r="AI78" t="inlineStr"/>
+      <c r="AI78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 43, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AJ78" t="inlineStr"/>
       <c r="AK78" t="inlineStr"/>
       <c r="AL78" t="inlineStr"/>
       <c r="AM78" t="inlineStr"/>
-      <c r="AN78" t="inlineStr"/>
-      <c r="AO78" t="inlineStr"/>
+      <c r="AN78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="AO78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+</t>
+        </is>
+      </c>
       <c r="AP78" t="inlineStr"/>
       <c r="AQ78" t="inlineStr"/>
-      <c r="AR78" t="inlineStr"/>
+      <c r="AR78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AS78" t="inlineStr"/>
       <c r="AT78" t="inlineStr"/>
-      <c r="AU78" t="inlineStr"/>
+      <c r="AU78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV78" t="inlineStr"/>
       <c r="AW78" t="inlineStr"/>
     </row>
@@ -4344,47 +4895,116 @@
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr"/>
       <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr"/>
-      <c r="T81" t="inlineStr"/>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U81" t="inlineStr"/>
       <c r="V81" t="inlineStr"/>
       <c r="W81" t="inlineStr"/>
-      <c r="X81" t="inlineStr"/>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y81" t="inlineStr"/>
       <c r="Z81" t="inlineStr"/>
-      <c r="AA81" t="inlineStr"/>
-      <c r="AB81" t="inlineStr"/>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 25, 6];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 25, 16];
+</t>
+        </is>
+      </c>
+      <c r="AB81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 26, 15];
+</t>
+        </is>
+      </c>
       <c r="AC81" t="inlineStr"/>
       <c r="AD81" t="inlineStr"/>
-      <c r="AE81" t="inlineStr"/>
+      <c r="AE81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11];
+</t>
+        </is>
+      </c>
       <c r="AF81" t="inlineStr"/>
       <c r="AG81" t="inlineStr"/>
       <c r="AH81" t="inlineStr"/>
-      <c r="AI81" t="inlineStr"/>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 43, 13, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AJ81" t="inlineStr"/>
       <c r="AK81" t="inlineStr"/>
       <c r="AL81" t="inlineStr"/>
       <c r="AM81" t="inlineStr"/>
       <c r="AN81" t="inlineStr"/>
-      <c r="AO81" t="inlineStr"/>
+      <c r="AO81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP81" t="inlineStr"/>
       <c r="AQ81" t="inlineStr"/>
       <c r="AR81" t="inlineStr"/>
-      <c r="AS81" t="inlineStr"/>
+      <c r="AS81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 43, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 43, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AT81" t="inlineStr"/>
-      <c r="AU81" t="inlineStr"/>
+      <c r="AU81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV81" t="inlineStr"/>
       <c r="AW81" t="inlineStr"/>
     </row>
@@ -4461,24 +5081,74 @@
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 25, 6, 23];
+data:[31, 37, 40, 22, 18, 45, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 28];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 41];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 30];
+</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 43, 13, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="P84" t="inlineStr"/>
       <c r="Q84" t="inlineStr"/>
-      <c r="R84" t="inlineStr"/>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 25, 16, 23];
+</t>
+        </is>
+      </c>
       <c r="S84" t="inlineStr"/>
-      <c r="T84" t="inlineStr"/>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U84" t="inlineStr"/>
       <c r="V84" t="inlineStr"/>
       <c r="W84" t="inlineStr"/>
-      <c r="X84" t="inlineStr"/>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y84" t="inlineStr"/>
       <c r="Z84" t="inlineStr"/>
       <c r="AA84" t="inlineStr"/>
@@ -4495,13 +5165,24 @@
       <c r="AL84" t="inlineStr"/>
       <c r="AM84" t="inlineStr"/>
       <c r="AN84" t="inlineStr"/>
-      <c r="AO84" t="inlineStr"/>
+      <c r="AO84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP84" t="inlineStr"/>
       <c r="AQ84" t="inlineStr"/>
       <c r="AR84" t="inlineStr"/>
       <c r="AS84" t="inlineStr"/>
       <c r="AT84" t="inlineStr"/>
-      <c r="AU84" t="inlineStr"/>
+      <c r="AU84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV84" t="inlineStr"/>
       <c r="AW84" t="inlineStr"/>
     </row>
@@ -4578,10 +5259,20 @@
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr"/>
@@ -4591,19 +5282,49 @@
       <c r="Q87" t="inlineStr"/>
       <c r="R87" t="inlineStr"/>
       <c r="S87" t="inlineStr"/>
-      <c r="T87" t="inlineStr"/>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U87" t="inlineStr"/>
       <c r="V87" t="inlineStr"/>
       <c r="W87" t="inlineStr"/>
-      <c r="X87" t="inlineStr"/>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y87" t="inlineStr"/>
       <c r="Z87" t="inlineStr"/>
-      <c r="AA87" t="inlineStr"/>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 25, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AB87" t="inlineStr"/>
       <c r="AC87" t="inlineStr"/>
-      <c r="AD87" t="inlineStr"/>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 28, 3];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 28, 7];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 28, 41];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 28, 30];
+</t>
+        </is>
+      </c>
       <c r="AE87" t="inlineStr"/>
-      <c r="AF87" t="inlineStr"/>
+      <c r="AF87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 30, 28];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 30, 41];
+</t>
+        </is>
+      </c>
       <c r="AG87" t="inlineStr"/>
       <c r="AH87" t="inlineStr"/>
       <c r="AI87" t="inlineStr"/>
@@ -4611,15 +5332,45 @@
       <c r="AK87" t="inlineStr"/>
       <c r="AL87" t="inlineStr"/>
       <c r="AM87" t="inlineStr"/>
-      <c r="AN87" t="inlineStr"/>
-      <c r="AO87" t="inlineStr"/>
+      <c r="AN87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
+      <c r="AO87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP87" t="inlineStr"/>
-      <c r="AQ87" t="inlineStr"/>
+      <c r="AQ87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 41, 3];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 41, 28];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 41, 30];
+</t>
+        </is>
+      </c>
       <c r="AR87" t="inlineStr"/>
       <c r="AS87" t="inlineStr"/>
       <c r="AT87" t="inlineStr"/>
-      <c r="AU87" t="inlineStr"/>
-      <c r="AV87" t="inlineStr"/>
+      <c r="AU87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
+      <c r="AV87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46, 3];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46, 7];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46, 34];
+</t>
+        </is>
+      </c>
       <c r="AW87" t="inlineStr"/>
     </row>
     <row r="88">
@@ -4693,26 +5444,71 @@
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 41, 3, 46];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 41, 3, 17];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 41, 3, 19];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 41, 3, 28];
+</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46, 7, 28];
+</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 25, 6, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 26, 15, 25, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="R90" t="inlineStr"/>
       <c r="S90" t="inlineStr"/>
-      <c r="T90" t="inlineStr"/>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U90" t="inlineStr"/>
-      <c r="V90" t="inlineStr"/>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="W90" t="inlineStr"/>
-      <c r="X90" t="inlineStr"/>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y90" t="inlineStr"/>
       <c r="Z90" t="inlineStr"/>
       <c r="AA90" t="inlineStr"/>
@@ -4724,18 +5520,36 @@
       <c r="AG90" t="inlineStr"/>
       <c r="AH90" t="inlineStr"/>
       <c r="AI90" t="inlineStr"/>
-      <c r="AJ90" t="inlineStr"/>
+      <c r="AJ90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46, 34, 32];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46, 34, 35];
+rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46, 34, 44];
+</t>
+        </is>
+      </c>
       <c r="AK90" t="inlineStr"/>
       <c r="AL90" t="inlineStr"/>
       <c r="AM90" t="inlineStr"/>
       <c r="AN90" t="inlineStr"/>
-      <c r="AO90" t="inlineStr"/>
+      <c r="AO90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP90" t="inlineStr"/>
       <c r="AQ90" t="inlineStr"/>
       <c r="AR90" t="inlineStr"/>
       <c r="AS90" t="inlineStr"/>
       <c r="AT90" t="inlineStr"/>
-      <c r="AU90" t="inlineStr"/>
+      <c r="AU90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV90" t="inlineStr"/>
       <c r="AW90" t="inlineStr"/>
     </row>
@@ -4812,10 +5626,20 @@
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24];
+</t>
+        </is>
+      </c>
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
@@ -4825,15 +5649,32 @@
       <c r="Q93" t="inlineStr"/>
       <c r="R93" t="inlineStr"/>
       <c r="S93" t="inlineStr"/>
-      <c r="T93" t="inlineStr"/>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U93" t="inlineStr"/>
       <c r="V93" t="inlineStr"/>
       <c r="W93" t="inlineStr"/>
-      <c r="X93" t="inlineStr"/>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y93" t="inlineStr"/>
       <c r="Z93" t="inlineStr"/>
       <c r="AA93" t="inlineStr"/>
-      <c r="AB93" t="inlineStr"/>
+      <c r="AB93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 12, 26, 15, 25, 6, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 38, 15, 26, 15, 25, 6, 23];
+</t>
+        </is>
+      </c>
       <c r="AC93" t="inlineStr"/>
       <c r="AD93" t="inlineStr"/>
       <c r="AE93" t="inlineStr"/>
@@ -4846,13 +5687,29 @@
       <c r="AL93" t="inlineStr"/>
       <c r="AM93" t="inlineStr"/>
       <c r="AN93" t="inlineStr"/>
-      <c r="AO93" t="inlineStr"/>
+      <c r="AO93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP93" t="inlineStr"/>
       <c r="AQ93" t="inlineStr"/>
       <c r="AR93" t="inlineStr"/>
       <c r="AS93" t="inlineStr"/>
-      <c r="AT93" t="inlineStr"/>
-      <c r="AU93" t="inlineStr"/>
+      <c r="AT93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 29, 11, 46, 34, 44, 36];
+</t>
+        </is>
+      </c>
+      <c r="AU93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV93" t="inlineStr"/>
       <c r="AW93" t="inlineStr"/>
     </row>
@@ -4929,7 +5786,12 @@
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
@@ -4942,13 +5804,29 @@
       <c r="Q96" t="inlineStr"/>
       <c r="R96" t="inlineStr"/>
       <c r="S96" t="inlineStr"/>
-      <c r="T96" t="inlineStr"/>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U96" t="inlineStr"/>
       <c r="V96" t="inlineStr"/>
       <c r="W96" t="inlineStr"/>
-      <c r="X96" t="inlineStr"/>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y96" t="inlineStr"/>
-      <c r="Z96" t="inlineStr"/>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24, 5];
+</t>
+        </is>
+      </c>
       <c r="AA96" t="inlineStr"/>
       <c r="AB96" t="inlineStr"/>
       <c r="AC96" t="inlineStr"/>
@@ -4963,13 +5841,24 @@
       <c r="AL96" t="inlineStr"/>
       <c r="AM96" t="inlineStr"/>
       <c r="AN96" t="inlineStr"/>
-      <c r="AO96" t="inlineStr"/>
+      <c r="AO96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP96" t="inlineStr"/>
       <c r="AQ96" t="inlineStr"/>
       <c r="AR96" t="inlineStr"/>
       <c r="AS96" t="inlineStr"/>
       <c r="AT96" t="inlineStr"/>
-      <c r="AU96" t="inlineStr"/>
+      <c r="AU96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV96" t="inlineStr"/>
       <c r="AW96" t="inlineStr"/>
     </row>
@@ -5046,7 +5935,12 @@
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
@@ -5059,13 +5953,29 @@
       <c r="Q99" t="inlineStr"/>
       <c r="R99" t="inlineStr"/>
       <c r="S99" t="inlineStr"/>
-      <c r="T99" t="inlineStr"/>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U99" t="inlineStr"/>
       <c r="V99" t="inlineStr"/>
       <c r="W99" t="inlineStr"/>
-      <c r="X99" t="inlineStr"/>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y99" t="inlineStr"/>
-      <c r="Z99" t="inlineStr"/>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24, 5];
+</t>
+        </is>
+      </c>
       <c r="AA99" t="inlineStr"/>
       <c r="AB99" t="inlineStr"/>
       <c r="AC99" t="inlineStr"/>
@@ -5080,13 +5990,24 @@
       <c r="AL99" t="inlineStr"/>
       <c r="AM99" t="inlineStr"/>
       <c r="AN99" t="inlineStr"/>
-      <c r="AO99" t="inlineStr"/>
+      <c r="AO99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP99" t="inlineStr"/>
       <c r="AQ99" t="inlineStr"/>
       <c r="AR99" t="inlineStr"/>
       <c r="AS99" t="inlineStr"/>
       <c r="AT99" t="inlineStr"/>
-      <c r="AU99" t="inlineStr"/>
+      <c r="AU99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV99" t="inlineStr"/>
       <c r="AW99" t="inlineStr"/>
     </row>
@@ -5163,7 +6084,12 @@
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr"/>
@@ -5176,13 +6102,29 @@
       <c r="Q102" t="inlineStr"/>
       <c r="R102" t="inlineStr"/>
       <c r="S102" t="inlineStr"/>
-      <c r="T102" t="inlineStr"/>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U102" t="inlineStr"/>
       <c r="V102" t="inlineStr"/>
       <c r="W102" t="inlineStr"/>
-      <c r="X102" t="inlineStr"/>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y102" t="inlineStr"/>
-      <c r="Z102" t="inlineStr"/>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24, 5];
+</t>
+        </is>
+      </c>
       <c r="AA102" t="inlineStr"/>
       <c r="AB102" t="inlineStr"/>
       <c r="AC102" t="inlineStr"/>
@@ -5197,13 +6139,24 @@
       <c r="AL102" t="inlineStr"/>
       <c r="AM102" t="inlineStr"/>
       <c r="AN102" t="inlineStr"/>
-      <c r="AO102" t="inlineStr"/>
+      <c r="AO102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP102" t="inlineStr"/>
       <c r="AQ102" t="inlineStr"/>
       <c r="AR102" t="inlineStr"/>
       <c r="AS102" t="inlineStr"/>
       <c r="AT102" t="inlineStr"/>
-      <c r="AU102" t="inlineStr"/>
+      <c r="AU102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV102" t="inlineStr"/>
       <c r="AW102" t="inlineStr"/>
     </row>
@@ -5280,7 +6233,12 @@
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 18, 45, 20, 39, 5, 24];
+</t>
+        </is>
+      </c>
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
@@ -5293,13 +6251,29 @@
       <c r="Q105" t="inlineStr"/>
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr"/>
-      <c r="T105" t="inlineStr"/>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U105" t="inlineStr"/>
       <c r="V105" t="inlineStr"/>
       <c r="W105" t="inlineStr"/>
-      <c r="X105" t="inlineStr"/>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+rreg:[31, 37, 40, 22, 8];
+</t>
+        </is>
+      </c>
       <c r="Y105" t="inlineStr"/>
-      <c r="Z105" t="inlineStr"/>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24, 5];
+</t>
+        </is>
+      </c>
       <c r="AA105" t="inlineStr"/>
       <c r="AB105" t="inlineStr"/>
       <c r="AC105" t="inlineStr"/>
@@ -5314,13 +6288,24 @@
       <c r="AL105" t="inlineStr"/>
       <c r="AM105" t="inlineStr"/>
       <c r="AN105" t="inlineStr"/>
-      <c r="AO105" t="inlineStr"/>
+      <c r="AO105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP105" t="inlineStr"/>
       <c r="AQ105" t="inlineStr"/>
       <c r="AR105" t="inlineStr"/>
       <c r="AS105" t="inlineStr"/>
       <c r="AT105" t="inlineStr"/>
-      <c r="AU105" t="inlineStr"/>
+      <c r="AU105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV105" t="inlineStr"/>
       <c r="AW105" t="inlineStr"/>
     </row>
@@ -5410,13 +6395,28 @@
       <c r="Q108" t="inlineStr"/>
       <c r="R108" t="inlineStr"/>
       <c r="S108" t="inlineStr"/>
-      <c r="T108" t="inlineStr"/>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U108" t="inlineStr"/>
       <c r="V108" t="inlineStr"/>
       <c r="W108" t="inlineStr"/>
-      <c r="X108" t="inlineStr"/>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 5];
+</t>
+        </is>
+      </c>
       <c r="Y108" t="inlineStr"/>
-      <c r="Z108" t="inlineStr"/>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24, 5];
+</t>
+        </is>
+      </c>
       <c r="AA108" t="inlineStr"/>
       <c r="AB108" t="inlineStr"/>
       <c r="AC108" t="inlineStr"/>
@@ -5431,13 +6431,24 @@
       <c r="AL108" t="inlineStr"/>
       <c r="AM108" t="inlineStr"/>
       <c r="AN108" t="inlineStr"/>
-      <c r="AO108" t="inlineStr"/>
+      <c r="AO108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP108" t="inlineStr"/>
       <c r="AQ108" t="inlineStr"/>
       <c r="AR108" t="inlineStr"/>
       <c r="AS108" t="inlineStr"/>
       <c r="AT108" t="inlineStr"/>
-      <c r="AU108" t="inlineStr"/>
+      <c r="AU108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV108" t="inlineStr"/>
       <c r="AW108" t="inlineStr"/>
     </row>
@@ -5527,13 +6538,23 @@
       <c r="Q111" t="inlineStr"/>
       <c r="R111" t="inlineStr"/>
       <c r="S111" t="inlineStr"/>
-      <c r="T111" t="inlineStr"/>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U111" t="inlineStr"/>
       <c r="V111" t="inlineStr"/>
       <c r="W111" t="inlineStr"/>
       <c r="X111" t="inlineStr"/>
       <c r="Y111" t="inlineStr"/>
-      <c r="Z111" t="inlineStr"/>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 24, 5];
+</t>
+        </is>
+      </c>
       <c r="AA111" t="inlineStr"/>
       <c r="AB111" t="inlineStr"/>
       <c r="AC111" t="inlineStr"/>
@@ -5548,13 +6569,24 @@
       <c r="AL111" t="inlineStr"/>
       <c r="AM111" t="inlineStr"/>
       <c r="AN111" t="inlineStr"/>
-      <c r="AO111" t="inlineStr"/>
+      <c r="AO111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP111" t="inlineStr"/>
       <c r="AQ111" t="inlineStr"/>
       <c r="AR111" t="inlineStr"/>
       <c r="AS111" t="inlineStr"/>
       <c r="AT111" t="inlineStr"/>
-      <c r="AU111" t="inlineStr"/>
+      <c r="AU111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV111" t="inlineStr"/>
       <c r="AW111" t="inlineStr"/>
     </row>
@@ -5644,7 +6676,12 @@
       <c r="Q114" t="inlineStr"/>
       <c r="R114" t="inlineStr"/>
       <c r="S114" t="inlineStr"/>
-      <c r="T114" t="inlineStr"/>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U114" t="inlineStr"/>
       <c r="V114" t="inlineStr"/>
       <c r="W114" t="inlineStr"/>
@@ -5665,13 +6702,24 @@
       <c r="AL114" t="inlineStr"/>
       <c r="AM114" t="inlineStr"/>
       <c r="AN114" t="inlineStr"/>
-      <c r="AO114" t="inlineStr"/>
+      <c r="AO114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP114" t="inlineStr"/>
       <c r="AQ114" t="inlineStr"/>
       <c r="AR114" t="inlineStr"/>
       <c r="AS114" t="inlineStr"/>
       <c r="AT114" t="inlineStr"/>
-      <c r="AU114" t="inlineStr"/>
+      <c r="AU114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV114" t="inlineStr"/>
       <c r="AW114" t="inlineStr"/>
     </row>
@@ -5761,7 +6809,12 @@
       <c r="Q117" t="inlineStr"/>
       <c r="R117" t="inlineStr"/>
       <c r="S117" t="inlineStr"/>
-      <c r="T117" t="inlineStr"/>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U117" t="inlineStr"/>
       <c r="V117" t="inlineStr"/>
       <c r="W117" t="inlineStr"/>
@@ -5782,13 +6835,24 @@
       <c r="AL117" t="inlineStr"/>
       <c r="AM117" t="inlineStr"/>
       <c r="AN117" t="inlineStr"/>
-      <c r="AO117" t="inlineStr"/>
+      <c r="AO117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP117" t="inlineStr"/>
       <c r="AQ117" t="inlineStr"/>
       <c r="AR117" t="inlineStr"/>
       <c r="AS117" t="inlineStr"/>
       <c r="AT117" t="inlineStr"/>
-      <c r="AU117" t="inlineStr"/>
+      <c r="AU117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 5];
+</t>
+        </is>
+      </c>
       <c r="AV117" t="inlineStr"/>
       <c r="AW117" t="inlineStr"/>
     </row>
@@ -5878,7 +6942,12 @@
       <c r="Q120" t="inlineStr"/>
       <c r="R120" t="inlineStr"/>
       <c r="S120" t="inlineStr"/>
-      <c r="T120" t="inlineStr"/>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U120" t="inlineStr"/>
       <c r="V120" t="inlineStr"/>
       <c r="W120" t="inlineStr"/>
@@ -5899,7 +6968,13 @@
       <c r="AL120" t="inlineStr"/>
       <c r="AM120" t="inlineStr"/>
       <c r="AN120" t="inlineStr"/>
-      <c r="AO120" t="inlineStr"/>
+      <c r="AO120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP120" t="inlineStr"/>
       <c r="AQ120" t="inlineStr"/>
       <c r="AR120" t="inlineStr"/>
@@ -5995,7 +7070,12 @@
       <c r="Q123" t="inlineStr"/>
       <c r="R123" t="inlineStr"/>
       <c r="S123" t="inlineStr"/>
-      <c r="T123" t="inlineStr"/>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U123" t="inlineStr"/>
       <c r="V123" t="inlineStr"/>
       <c r="W123" t="inlineStr"/>
@@ -6016,7 +7096,13 @@
       <c r="AL123" t="inlineStr"/>
       <c r="AM123" t="inlineStr"/>
       <c r="AN123" t="inlineStr"/>
-      <c r="AO123" t="inlineStr"/>
+      <c r="AO123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP123" t="inlineStr"/>
       <c r="AQ123" t="inlineStr"/>
       <c r="AR123" t="inlineStr"/>
@@ -6112,7 +7198,12 @@
       <c r="Q126" t="inlineStr"/>
       <c r="R126" t="inlineStr"/>
       <c r="S126" t="inlineStr"/>
-      <c r="T126" t="inlineStr"/>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U126" t="inlineStr"/>
       <c r="V126" t="inlineStr"/>
       <c r="W126" t="inlineStr"/>
@@ -6133,7 +7224,13 @@
       <c r="AL126" t="inlineStr"/>
       <c r="AM126" t="inlineStr"/>
       <c r="AN126" t="inlineStr"/>
-      <c r="AO126" t="inlineStr"/>
+      <c r="AO126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP126" t="inlineStr"/>
       <c r="AQ126" t="inlineStr"/>
       <c r="AR126" t="inlineStr"/>
@@ -6229,7 +7326,12 @@
       <c r="Q129" t="inlineStr"/>
       <c r="R129" t="inlineStr"/>
       <c r="S129" t="inlineStr"/>
-      <c r="T129" t="inlineStr"/>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U129" t="inlineStr"/>
       <c r="V129" t="inlineStr"/>
       <c r="W129" t="inlineStr"/>
@@ -6250,7 +7352,13 @@
       <c r="AL129" t="inlineStr"/>
       <c r="AM129" t="inlineStr"/>
       <c r="AN129" t="inlineStr"/>
-      <c r="AO129" t="inlineStr"/>
+      <c r="AO129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP129" t="inlineStr"/>
       <c r="AQ129" t="inlineStr"/>
       <c r="AR129" t="inlineStr"/>
@@ -6346,7 +7454,12 @@
       <c r="Q132" t="inlineStr"/>
       <c r="R132" t="inlineStr"/>
       <c r="S132" t="inlineStr"/>
-      <c r="T132" t="inlineStr"/>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U132" t="inlineStr"/>
       <c r="V132" t="inlineStr"/>
       <c r="W132" t="inlineStr"/>
@@ -6367,7 +7480,13 @@
       <c r="AL132" t="inlineStr"/>
       <c r="AM132" t="inlineStr"/>
       <c r="AN132" t="inlineStr"/>
-      <c r="AO132" t="inlineStr"/>
+      <c r="AO132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP132" t="inlineStr"/>
       <c r="AQ132" t="inlineStr"/>
       <c r="AR132" t="inlineStr"/>
@@ -6463,7 +7582,12 @@
       <c r="Q135" t="inlineStr"/>
       <c r="R135" t="inlineStr"/>
       <c r="S135" t="inlineStr"/>
-      <c r="T135" t="inlineStr"/>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U135" t="inlineStr"/>
       <c r="V135" t="inlineStr"/>
       <c r="W135" t="inlineStr"/>
@@ -6484,7 +7608,13 @@
       <c r="AL135" t="inlineStr"/>
       <c r="AM135" t="inlineStr"/>
       <c r="AN135" t="inlineStr"/>
-      <c r="AO135" t="inlineStr"/>
+      <c r="AO135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP135" t="inlineStr"/>
       <c r="AQ135" t="inlineStr"/>
       <c r="AR135" t="inlineStr"/>
@@ -6580,7 +7710,12 @@
       <c r="Q138" t="inlineStr"/>
       <c r="R138" t="inlineStr"/>
       <c r="S138" t="inlineStr"/>
-      <c r="T138" t="inlineStr"/>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U138" t="inlineStr"/>
       <c r="V138" t="inlineStr"/>
       <c r="W138" t="inlineStr"/>
@@ -6601,7 +7736,13 @@
       <c r="AL138" t="inlineStr"/>
       <c r="AM138" t="inlineStr"/>
       <c r="AN138" t="inlineStr"/>
-      <c r="AO138" t="inlineStr"/>
+      <c r="AO138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP138" t="inlineStr"/>
       <c r="AQ138" t="inlineStr"/>
       <c r="AR138" t="inlineStr"/>
@@ -6697,7 +7838,12 @@
       <c r="Q141" t="inlineStr"/>
       <c r="R141" t="inlineStr"/>
       <c r="S141" t="inlineStr"/>
-      <c r="T141" t="inlineStr"/>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U141" t="inlineStr"/>
       <c r="V141" t="inlineStr"/>
       <c r="W141" t="inlineStr"/>
@@ -6718,7 +7864,13 @@
       <c r="AL141" t="inlineStr"/>
       <c r="AM141" t="inlineStr"/>
       <c r="AN141" t="inlineStr"/>
-      <c r="AO141" t="inlineStr"/>
+      <c r="AO141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP141" t="inlineStr"/>
       <c r="AQ141" t="inlineStr"/>
       <c r="AR141" t="inlineStr"/>
@@ -6814,7 +7966,12 @@
       <c r="Q144" t="inlineStr"/>
       <c r="R144" t="inlineStr"/>
       <c r="S144" t="inlineStr"/>
-      <c r="T144" t="inlineStr"/>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U144" t="inlineStr"/>
       <c r="V144" t="inlineStr"/>
       <c r="W144" t="inlineStr"/>
@@ -6835,7 +7992,13 @@
       <c r="AL144" t="inlineStr"/>
       <c r="AM144" t="inlineStr"/>
       <c r="AN144" t="inlineStr"/>
-      <c r="AO144" t="inlineStr"/>
+      <c r="AO144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP144" t="inlineStr"/>
       <c r="AQ144" t="inlineStr"/>
       <c r="AR144" t="inlineStr"/>
@@ -6931,7 +8094,12 @@
       <c r="Q147" t="inlineStr"/>
       <c r="R147" t="inlineStr"/>
       <c r="S147" t="inlineStr"/>
-      <c r="T147" t="inlineStr"/>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 20, 45, 18, 5];
+</t>
+        </is>
+      </c>
       <c r="U147" t="inlineStr"/>
       <c r="V147" t="inlineStr"/>
       <c r="W147" t="inlineStr"/>
@@ -6952,7 +8120,13 @@
       <c r="AL147" t="inlineStr"/>
       <c r="AM147" t="inlineStr"/>
       <c r="AN147" t="inlineStr"/>
-      <c r="AO147" t="inlineStr"/>
+      <c r="AO147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP147" t="inlineStr"/>
       <c r="AQ147" t="inlineStr"/>
       <c r="AR147" t="inlineStr"/>
@@ -7069,7 +8243,13 @@
       <c r="AL150" t="inlineStr"/>
       <c r="AM150" t="inlineStr"/>
       <c r="AN150" t="inlineStr"/>
-      <c r="AO150" t="inlineStr"/>
+      <c r="AO150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP150" t="inlineStr"/>
       <c r="AQ150" t="inlineStr"/>
       <c r="AR150" t="inlineStr"/>
@@ -7186,7 +8366,13 @@
       <c r="AL153" t="inlineStr"/>
       <c r="AM153" t="inlineStr"/>
       <c r="AN153" t="inlineStr"/>
-      <c r="AO153" t="inlineStr"/>
+      <c r="AO153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rreg:[31, 37, 40, 22, 21, 8, 39, 5];
+rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP153" t="inlineStr"/>
       <c r="AQ153" t="inlineStr"/>
       <c r="AR153" t="inlineStr"/>
@@ -7303,7 +8489,12 @@
       <c r="AL156" t="inlineStr"/>
       <c r="AM156" t="inlineStr"/>
       <c r="AN156" t="inlineStr"/>
-      <c r="AO156" t="inlineStr"/>
+      <c r="AO156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP156" t="inlineStr"/>
       <c r="AQ156" t="inlineStr"/>
       <c r="AR156" t="inlineStr"/>
@@ -7420,7 +8611,12 @@
       <c r="AL159" t="inlineStr"/>
       <c r="AM159" t="inlineStr"/>
       <c r="AN159" t="inlineStr"/>
-      <c r="AO159" t="inlineStr"/>
+      <c r="AO159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP159" t="inlineStr"/>
       <c r="AQ159" t="inlineStr"/>
       <c r="AR159" t="inlineStr"/>
@@ -7537,7 +8733,12 @@
       <c r="AL162" t="inlineStr"/>
       <c r="AM162" t="inlineStr"/>
       <c r="AN162" t="inlineStr"/>
-      <c r="AO162" t="inlineStr"/>
+      <c r="AO162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP162" t="inlineStr"/>
       <c r="AQ162" t="inlineStr"/>
       <c r="AR162" t="inlineStr"/>
@@ -7654,7 +8855,12 @@
       <c r="AL165" t="inlineStr"/>
       <c r="AM165" t="inlineStr"/>
       <c r="AN165" t="inlineStr"/>
-      <c r="AO165" t="inlineStr"/>
+      <c r="AO165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP165" t="inlineStr"/>
       <c r="AQ165" t="inlineStr"/>
       <c r="AR165" t="inlineStr"/>
@@ -7771,7 +8977,12 @@
       <c r="AL168" t="inlineStr"/>
       <c r="AM168" t="inlineStr"/>
       <c r="AN168" t="inlineStr"/>
-      <c r="AO168" t="inlineStr"/>
+      <c r="AO168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP168" t="inlineStr"/>
       <c r="AQ168" t="inlineStr"/>
       <c r="AR168" t="inlineStr"/>
@@ -7888,7 +9099,12 @@
       <c r="AL171" t="inlineStr"/>
       <c r="AM171" t="inlineStr"/>
       <c r="AN171" t="inlineStr"/>
-      <c r="AO171" t="inlineStr"/>
+      <c r="AO171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP171" t="inlineStr"/>
       <c r="AQ171" t="inlineStr"/>
       <c r="AR171" t="inlineStr"/>
@@ -8005,7 +9221,12 @@
       <c r="AL174" t="inlineStr"/>
       <c r="AM174" t="inlineStr"/>
       <c r="AN174" t="inlineStr"/>
-      <c r="AO174" t="inlineStr"/>
+      <c r="AO174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP174" t="inlineStr"/>
       <c r="AQ174" t="inlineStr"/>
       <c r="AR174" t="inlineStr"/>
@@ -8122,7 +9343,12 @@
       <c r="AL177" t="inlineStr"/>
       <c r="AM177" t="inlineStr"/>
       <c r="AN177" t="inlineStr"/>
-      <c r="AO177" t="inlineStr"/>
+      <c r="AO177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP177" t="inlineStr"/>
       <c r="AQ177" t="inlineStr"/>
       <c r="AR177" t="inlineStr"/>
@@ -8239,7 +9465,12 @@
       <c r="AL180" t="inlineStr"/>
       <c r="AM180" t="inlineStr"/>
       <c r="AN180" t="inlineStr"/>
-      <c r="AO180" t="inlineStr"/>
+      <c r="AO180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP180" t="inlineStr"/>
       <c r="AQ180" t="inlineStr"/>
       <c r="AR180" t="inlineStr"/>
@@ -8356,7 +9587,12 @@
       <c r="AL183" t="inlineStr"/>
       <c r="AM183" t="inlineStr"/>
       <c r="AN183" t="inlineStr"/>
-      <c r="AO183" t="inlineStr"/>
+      <c r="AO183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP183" t="inlineStr"/>
       <c r="AQ183" t="inlineStr"/>
       <c r="AR183" t="inlineStr"/>
@@ -8473,7 +9709,12 @@
       <c r="AL186" t="inlineStr"/>
       <c r="AM186" t="inlineStr"/>
       <c r="AN186" t="inlineStr"/>
-      <c r="AO186" t="inlineStr"/>
+      <c r="AO186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP186" t="inlineStr"/>
       <c r="AQ186" t="inlineStr"/>
       <c r="AR186" t="inlineStr"/>
@@ -8590,7 +9831,12 @@
       <c r="AL189" t="inlineStr"/>
       <c r="AM189" t="inlineStr"/>
       <c r="AN189" t="inlineStr"/>
-      <c r="AO189" t="inlineStr"/>
+      <c r="AO189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AP189" t="inlineStr"/>
       <c r="AQ189" t="inlineStr"/>
       <c r="AR189" t="inlineStr"/>
@@ -8676,7 +9922,15 @@
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr"/>
-      <c r="J192" t="inlineStr"/>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K192" t="inlineStr"/>
       <c r="L192" t="inlineStr"/>
       <c r="M192" t="inlineStr"/>
@@ -8793,7 +10047,15 @@
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr"/>
       <c r="I195" t="inlineStr"/>
-      <c r="J195" t="inlineStr"/>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K195" t="inlineStr"/>
       <c r="L195" t="inlineStr"/>
       <c r="M195" t="inlineStr"/>
@@ -8910,7 +10172,15 @@
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr"/>
-      <c r="J198" t="inlineStr"/>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K198" t="inlineStr"/>
       <c r="L198" t="inlineStr"/>
       <c r="M198" t="inlineStr"/>
@@ -9027,7 +10297,15 @@
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr"/>
-      <c r="J201" t="inlineStr"/>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K201" t="inlineStr"/>
       <c r="L201" t="inlineStr"/>
       <c r="M201" t="inlineStr"/>
@@ -9144,7 +10422,15 @@
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr"/>
       <c r="I204" t="inlineStr"/>
-      <c r="J204" t="inlineStr"/>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K204" t="inlineStr"/>
       <c r="L204" t="inlineStr"/>
       <c r="M204" t="inlineStr"/>
@@ -9261,7 +10547,15 @@
       <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr"/>
-      <c r="J207" t="inlineStr"/>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K207" t="inlineStr"/>
       <c r="L207" t="inlineStr"/>
       <c r="M207" t="inlineStr"/>
@@ -9378,7 +10672,15 @@
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr"/>
-      <c r="J210" t="inlineStr"/>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K210" t="inlineStr"/>
       <c r="L210" t="inlineStr"/>
       <c r="M210" t="inlineStr"/>
@@ -9495,7 +10797,15 @@
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr"/>
       <c r="I213" t="inlineStr"/>
-      <c r="J213" t="inlineStr"/>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K213" t="inlineStr"/>
       <c r="L213" t="inlineStr"/>
       <c r="M213" t="inlineStr"/>
@@ -9612,7 +10922,14 @@
       <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr"/>
-      <c r="J216" t="inlineStr"/>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K216" t="inlineStr"/>
       <c r="L216" t="inlineStr"/>
       <c r="M216" t="inlineStr"/>
@@ -9729,7 +11046,13 @@
       <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr"/>
       <c r="I219" t="inlineStr"/>
-      <c r="J219" t="inlineStr"/>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 18, 45, 20, 39, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K219" t="inlineStr"/>
       <c r="L219" t="inlineStr"/>
       <c r="M219" t="inlineStr"/>
@@ -9846,7 +11169,12 @@
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr"/>
       <c r="I222" t="inlineStr"/>
-      <c r="J222" t="inlineStr"/>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K222" t="inlineStr"/>
       <c r="L222" t="inlineStr"/>
       <c r="M222" t="inlineStr"/>
@@ -9963,7 +11291,12 @@
       <c r="G225" t="inlineStr"/>
       <c r="H225" t="inlineStr"/>
       <c r="I225" t="inlineStr"/>
-      <c r="J225" t="inlineStr"/>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K225" t="inlineStr"/>
       <c r="L225" t="inlineStr"/>
       <c r="M225" t="inlineStr"/>
@@ -10080,7 +11413,12 @@
       <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr"/>
       <c r="I228" t="inlineStr"/>
-      <c r="J228" t="inlineStr"/>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K228" t="inlineStr"/>
       <c r="L228" t="inlineStr"/>
       <c r="M228" t="inlineStr"/>
@@ -10197,7 +11535,12 @@
       <c r="G231" t="inlineStr"/>
       <c r="H231" t="inlineStr"/>
       <c r="I231" t="inlineStr"/>
-      <c r="J231" t="inlineStr"/>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K231" t="inlineStr"/>
       <c r="L231" t="inlineStr"/>
       <c r="M231" t="inlineStr"/>
@@ -10314,7 +11657,12 @@
       <c r="G234" t="inlineStr"/>
       <c r="H234" t="inlineStr"/>
       <c r="I234" t="inlineStr"/>
-      <c r="J234" t="inlineStr"/>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K234" t="inlineStr"/>
       <c r="L234" t="inlineStr"/>
       <c r="M234" t="inlineStr"/>
@@ -10431,7 +11779,12 @@
       <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr"/>
       <c r="I237" t="inlineStr"/>
-      <c r="J237" t="inlineStr"/>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K237" t="inlineStr"/>
       <c r="L237" t="inlineStr"/>
       <c r="M237" t="inlineStr"/>
@@ -10548,7 +11901,12 @@
       <c r="G240" t="inlineStr"/>
       <c r="H240" t="inlineStr"/>
       <c r="I240" t="inlineStr"/>
-      <c r="J240" t="inlineStr"/>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K240" t="inlineStr"/>
       <c r="L240" t="inlineStr"/>
       <c r="M240" t="inlineStr"/>
@@ -10665,7 +12023,12 @@
       <c r="G243" t="inlineStr"/>
       <c r="H243" t="inlineStr"/>
       <c r="I243" t="inlineStr"/>
-      <c r="J243" t="inlineStr"/>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K243" t="inlineStr"/>
       <c r="L243" t="inlineStr"/>
       <c r="M243" t="inlineStr"/>
@@ -10782,7 +12145,12 @@
       <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr"/>
       <c r="I246" t="inlineStr"/>
-      <c r="J246" t="inlineStr"/>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K246" t="inlineStr"/>
       <c r="L246" t="inlineStr"/>
       <c r="M246" t="inlineStr"/>
@@ -10899,7 +12267,12 @@
       <c r="G249" t="inlineStr"/>
       <c r="H249" t="inlineStr"/>
       <c r="I249" t="inlineStr"/>
-      <c r="J249" t="inlineStr"/>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K249" t="inlineStr"/>
       <c r="L249" t="inlineStr"/>
       <c r="M249" t="inlineStr"/>
@@ -11016,7 +12389,12 @@
       <c r="G252" t="inlineStr"/>
       <c r="H252" t="inlineStr"/>
       <c r="I252" t="inlineStr"/>
-      <c r="J252" t="inlineStr"/>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K252" t="inlineStr"/>
       <c r="L252" t="inlineStr"/>
       <c r="M252" t="inlineStr"/>
@@ -11133,7 +12511,12 @@
       <c r="G255" t="inlineStr"/>
       <c r="H255" t="inlineStr"/>
       <c r="I255" t="inlineStr"/>
-      <c r="J255" t="inlineStr"/>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K255" t="inlineStr"/>
       <c r="L255" t="inlineStr"/>
       <c r="M255" t="inlineStr"/>
@@ -11250,7 +12633,12 @@
       <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr"/>
       <c r="I258" t="inlineStr"/>
-      <c r="J258" t="inlineStr"/>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K258" t="inlineStr"/>
       <c r="L258" t="inlineStr"/>
       <c r="M258" t="inlineStr"/>
@@ -11367,7 +12755,12 @@
       <c r="G261" t="inlineStr"/>
       <c r="H261" t="inlineStr"/>
       <c r="I261" t="inlineStr"/>
-      <c r="J261" t="inlineStr"/>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K261" t="inlineStr"/>
       <c r="L261" t="inlineStr"/>
       <c r="M261" t="inlineStr"/>
@@ -11484,7 +12877,12 @@
       <c r="G264" t="inlineStr"/>
       <c r="H264" t="inlineStr"/>
       <c r="I264" t="inlineStr"/>
-      <c r="J264" t="inlineStr"/>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K264" t="inlineStr"/>
       <c r="L264" t="inlineStr"/>
       <c r="M264" t="inlineStr"/>
@@ -11601,7 +12999,12 @@
       <c r="G267" t="inlineStr"/>
       <c r="H267" t="inlineStr"/>
       <c r="I267" t="inlineStr"/>
-      <c r="J267" t="inlineStr"/>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K267" t="inlineStr"/>
       <c r="L267" t="inlineStr"/>
       <c r="M267" t="inlineStr"/>
@@ -11718,7 +13121,12 @@
       <c r="G270" t="inlineStr"/>
       <c r="H270" t="inlineStr"/>
       <c r="I270" t="inlineStr"/>
-      <c r="J270" t="inlineStr"/>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K270" t="inlineStr"/>
       <c r="L270" t="inlineStr"/>
       <c r="M270" t="inlineStr"/>
@@ -11835,7 +13243,12 @@
       <c r="G273" t="inlineStr"/>
       <c r="H273" t="inlineStr"/>
       <c r="I273" t="inlineStr"/>
-      <c r="J273" t="inlineStr"/>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="K273" t="inlineStr"/>
       <c r="L273" t="inlineStr"/>
       <c r="M273" t="inlineStr"/>
@@ -11991,7 +13404,13 @@
       <c r="AT276" t="inlineStr"/>
       <c r="AU276" t="inlineStr"/>
       <c r="AV276" t="inlineStr"/>
-      <c r="AW276" t="inlineStr"/>
+      <c r="AW276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -12065,7 +13484,13 @@
       <c r="C279" t="inlineStr"/>
       <c r="D279" t="inlineStr"/>
       <c r="E279" t="inlineStr"/>
-      <c r="F279" t="inlineStr"/>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 18, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="G279" t="inlineStr"/>
       <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr"/>
@@ -12108,7 +13533,12 @@
       <c r="AT279" t="inlineStr"/>
       <c r="AU279" t="inlineStr"/>
       <c r="AV279" t="inlineStr"/>
-      <c r="AW279" t="inlineStr"/>
+      <c r="AW279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -12187,7 +13617,14 @@
       <c r="H282" t="inlineStr"/>
       <c r="I282" t="inlineStr"/>
       <c r="J282" t="inlineStr"/>
-      <c r="K282" t="inlineStr"/>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 27, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="L282" t="inlineStr"/>
       <c r="M282" t="inlineStr"/>
       <c r="N282" t="inlineStr"/>
@@ -12225,7 +13662,12 @@
       <c r="AT282" t="inlineStr"/>
       <c r="AU282" t="inlineStr"/>
       <c r="AV282" t="inlineStr"/>
-      <c r="AW282" t="inlineStr"/>
+      <c r="AW282" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -12297,7 +13739,13 @@
       </c>
       <c r="B285" t="inlineStr"/>
       <c r="C285" t="inlineStr"/>
-      <c r="D285" t="inlineStr"/>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 45, 2, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="E285" t="inlineStr"/>
       <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr"/>
@@ -12322,7 +13770,13 @@
       <c r="Z285" t="inlineStr"/>
       <c r="AA285" t="inlineStr"/>
       <c r="AB285" t="inlineStr"/>
-      <c r="AC285" t="inlineStr"/>
+      <c r="AC285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 27, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9, 27, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AD285" t="inlineStr"/>
       <c r="AE285" t="inlineStr"/>
       <c r="AF285" t="inlineStr"/>
@@ -12340,9 +13794,21 @@
       <c r="AR285" t="inlineStr"/>
       <c r="AS285" t="inlineStr"/>
       <c r="AT285" t="inlineStr"/>
-      <c r="AU285" t="inlineStr"/>
+      <c r="AU285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 39, 20, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 2, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+rrep:[31, 37, 40, 22, 21, 8, 39, 20, 2, 9, 45, 9, 4, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
       <c r="AV285" t="inlineStr"/>
-      <c r="AW285" t="inlineStr"/>
+      <c r="AW285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -12459,7 +13925,12 @@
       <c r="AT288" t="inlineStr"/>
       <c r="AU288" t="inlineStr"/>
       <c r="AV288" t="inlineStr"/>
-      <c r="AW288" t="inlineStr"/>
+      <c r="AW288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -12576,7 +14047,12 @@
       <c r="AT291" t="inlineStr"/>
       <c r="AU291" t="inlineStr"/>
       <c r="AV291" t="inlineStr"/>
-      <c r="AW291" t="inlineStr"/>
+      <c r="AW291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -12693,7 +14169,12 @@
       <c r="AT294" t="inlineStr"/>
       <c r="AU294" t="inlineStr"/>
       <c r="AV294" t="inlineStr"/>
-      <c r="AW294" t="inlineStr"/>
+      <c r="AW294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -12810,7 +14291,12 @@
       <c r="AT297" t="inlineStr"/>
       <c r="AU297" t="inlineStr"/>
       <c r="AV297" t="inlineStr"/>
-      <c r="AW297" t="inlineStr"/>
+      <c r="AW297" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -12927,7 +14413,12 @@
       <c r="AT300" t="inlineStr"/>
       <c r="AU300" t="inlineStr"/>
       <c r="AV300" t="inlineStr"/>
-      <c r="AW300" t="inlineStr"/>
+      <c r="AW300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -13044,7 +14535,12 @@
       <c r="AT303" t="inlineStr"/>
       <c r="AU303" t="inlineStr"/>
       <c r="AV303" t="inlineStr"/>
-      <c r="AW303" t="inlineStr"/>
+      <c r="AW303" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -13161,7 +14657,12 @@
       <c r="AT306" t="inlineStr"/>
       <c r="AU306" t="inlineStr"/>
       <c r="AV306" t="inlineStr"/>
-      <c r="AW306" t="inlineStr"/>
+      <c r="AW306" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -13278,7 +14779,12 @@
       <c r="AT309" t="inlineStr"/>
       <c r="AU309" t="inlineStr"/>
       <c r="AV309" t="inlineStr"/>
-      <c r="AW309" t="inlineStr"/>
+      <c r="AW309" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -13395,7 +14901,12 @@
       <c r="AT312" t="inlineStr"/>
       <c r="AU312" t="inlineStr"/>
       <c r="AV312" t="inlineStr"/>
-      <c r="AW312" t="inlineStr"/>
+      <c r="AW312" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -13512,7 +15023,12 @@
       <c r="AT315" t="inlineStr"/>
       <c r="AU315" t="inlineStr"/>
       <c r="AV315" t="inlineStr"/>
-      <c r="AW315" t="inlineStr"/>
+      <c r="AW315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -13629,7 +15145,12 @@
       <c r="AT318" t="inlineStr"/>
       <c r="AU318" t="inlineStr"/>
       <c r="AV318" t="inlineStr"/>
-      <c r="AW318" t="inlineStr"/>
+      <c r="AW318" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -13746,7 +15267,12 @@
       <c r="AT321" t="inlineStr"/>
       <c r="AU321" t="inlineStr"/>
       <c r="AV321" t="inlineStr"/>
-      <c r="AW321" t="inlineStr"/>
+      <c r="AW321" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -13863,7 +15389,12 @@
       <c r="AT324" t="inlineStr"/>
       <c r="AU324" t="inlineStr"/>
       <c r="AV324" t="inlineStr"/>
-      <c r="AW324" t="inlineStr"/>
+      <c r="AW324" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -13980,7 +15511,12 @@
       <c r="AT327" t="inlineStr"/>
       <c r="AU327" t="inlineStr"/>
       <c r="AV327" t="inlineStr"/>
-      <c r="AW327" t="inlineStr"/>
+      <c r="AW327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -14097,7 +15633,12 @@
       <c r="AT330" t="inlineStr"/>
       <c r="AU330" t="inlineStr"/>
       <c r="AV330" t="inlineStr"/>
-      <c r="AW330" t="inlineStr"/>
+      <c r="AW330" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rrep:[31, 37, 40, 22, 21, 8, 47, 8, 39, 42, 33, 23];
+</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">

</xml_diff>